<commit_message>
Corrige atualizacao das planilhas do dashboard
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\github_corrigido_dashboard_obrasRev1\github\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38D3F51D-200A-4500-8FFE-9E4651753B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D805BD9-6DCB-4FAA-87EB-09E91707409D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2879,7 +2879,7 @@
         <v>207.5</v>
       </c>
       <c r="F72" s="5">
-        <v>485.52</v>
+        <v>276.38</v>
       </c>
       <c r="I72">
         <v>1801</v>
@@ -2898,7 +2898,7 @@
       <c r="V72" s="4"/>
       <c r="W72" s="4"/>
       <c r="X72">
-        <v>485.52</v>
+        <v>276.38</v>
       </c>
       <c r="AG72" t="s">
         <v>114</v>

</xml_diff>

<commit_message>
Adiciona saldo por obra
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEE97603-A5C3-4271-951A-6B91FEF1BAE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEBF2523-B246-4AA1-AD38-80CDB183820F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -446,18 +446,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -472,7 +466,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -488,7 +482,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1612,7 +1605,7 @@
       </c>
     </row>
     <row r="10" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B10" t="s">
+      <c r="B10" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C10">
@@ -1669,7 +1662,7 @@
       </c>
     </row>
     <row r="11" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B11" t="s">
+      <c r="B11" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C11">
@@ -1707,7 +1700,7 @@
       </c>
     </row>
     <row r="12" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B12" t="s">
+      <c r="B12" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C12">
@@ -1758,7 +1751,7 @@
       </c>
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B13" t="s">
+      <c r="B13" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C13">
@@ -1799,7 +1792,7 @@
       </c>
     </row>
     <row r="14" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B14" t="s">
+      <c r="B14" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C14">
@@ -1812,7 +1805,8 @@
         <v>240.7</v>
       </c>
       <c r="F14" s="5">
-        <v>231.85</v>
+        <f>tb_base_dash_extensao[[#This Row],[produção Agosto 2025]]</f>
+        <v>159.47499999999999</v>
       </c>
       <c r="I14">
         <v>589</v>
@@ -1825,7 +1819,8 @@
       <c r="N14" s="6"/>
       <c r="O14" s="6"/>
       <c r="P14" s="8">
-        <v>231.85</v>
+        <f>231.85-72.375</f>
+        <v>159.47499999999999</v>
       </c>
       <c r="Q14" s="6"/>
       <c r="R14" s="6"/>
@@ -1848,7 +1843,7 @@
       </c>
     </row>
     <row r="15" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B15" t="s">
+      <c r="B15" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C15">
@@ -1891,7 +1886,7 @@
       </c>
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="B16" t="s">
+      <c r="B16" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C16">
@@ -1904,7 +1899,8 @@
         <v>0</v>
       </c>
       <c r="F16" s="5">
-        <v>367.71</v>
+        <f>tb_base_dash_extensao[[#This Row],[produção Agosto 2025]]+tb_base_dash_extensao[[#This Row],[produção Setembro 2025]]</f>
+        <v>295.33500000000004</v>
       </c>
       <c r="I16">
         <v>614</v>
@@ -1917,7 +1913,8 @@
       <c r="N16" s="6"/>
       <c r="O16" s="6"/>
       <c r="P16" s="8">
-        <v>132.27000000000001</v>
+        <f>132.27-72.375</f>
+        <v>59.89500000000001</v>
       </c>
       <c r="Q16" s="8">
         <v>235.44</v>
@@ -1942,7 +1939,7 @@
       </c>
     </row>
     <row r="17" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B17" t="s">
+      <c r="B17" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C17">
@@ -1959,9 +1956,7 @@
       <c r="N17" s="6"/>
       <c r="O17" s="6"/>
       <c r="P17" s="6"/>
-      <c r="Q17" s="9">
-        <v>154.93</v>
-      </c>
+      <c r="Q17" s="6"/>
       <c r="R17" s="6"/>
       <c r="S17" s="6"/>
       <c r="T17" s="6"/>
@@ -1982,7 +1977,7 @@
       </c>
     </row>
     <row r="18" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B18" t="s">
+      <c r="B18" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C18">
@@ -2031,7 +2026,7 @@
       </c>
     </row>
     <row r="19" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B19" t="s">
+      <c r="B19" s="5" t="s">
         <v>8</v>
       </c>
       <c r="C19">
@@ -2044,14 +2039,16 @@
         <v>754</v>
       </c>
       <c r="F19" s="5">
-        <v>445.46</v>
+        <f>tb_base_dash_extensao[[#This Row],[produção Agosto 2025]]+tb_base_dash_extensao[[#This Row],[produção Setembro 2025]]+tb_base_dash_extensao[[#This Row],[produção Dezembro 2025]]</f>
+        <v>373.08500000000004</v>
       </c>
       <c r="L19" s="6"/>
       <c r="M19" s="6"/>
       <c r="N19" s="6"/>
       <c r="O19" s="6"/>
       <c r="P19" s="6">
-        <v>242.97</v>
+        <f>242.97-72.375</f>
+        <v>170.595</v>
       </c>
       <c r="Q19" s="6">
         <v>148.49</v>

</xml_diff>

<commit_message>
Atualiza EAP de producao
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEBF2523-B246-4AA1-AD38-80CDB183820F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0181AE7C-595D-4014-9D5E-707E2A20A0F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9051,6 +9051,9 @@
       <c r="D192" t="s">
         <v>6</v>
       </c>
+      <c r="F192" s="5">
+        <v>78.19</v>
+      </c>
       <c r="L192" s="6"/>
       <c r="M192" s="6"/>
       <c r="N192" s="6"/>
@@ -9064,7 +9067,9 @@
       <c r="V192" s="6"/>
       <c r="W192" s="6"/>
       <c r="X192" s="6"/>
-      <c r="Y192" s="6"/>
+      <c r="Y192" s="6">
+        <v>78.19</v>
+      </c>
       <c r="Z192" s="6"/>
       <c r="AA192" s="6"/>
       <c r="AB192" s="6"/>

</xml_diff>

<commit_message>
Atualiza link do dashboard
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0181AE7C-595D-4014-9D5E-707E2A20A0F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DDC3DEE-9F23-4662-862F-278B02A0DDE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="121">
   <si>
     <t>Obra</t>
   </si>
@@ -397,6 +397,9 @@
   </si>
   <si>
     <t>CT LAGEADO MONTANTE</t>
+  </si>
+  <si>
+    <t>concuido</t>
   </si>
 </sst>
 </file>
@@ -7286,7 +7289,9 @@
       <c r="V145" s="6"/>
       <c r="W145" s="6"/>
       <c r="X145" s="6"/>
-      <c r="Y145" s="6"/>
+      <c r="Y145" s="6">
+        <v>42</v>
+      </c>
       <c r="Z145" s="6"/>
       <c r="AA145" s="6"/>
       <c r="AB145" s="6"/>
@@ -7700,7 +7705,7 @@
       <c r="AE156" s="6"/>
       <c r="AF156" s="6"/>
       <c r="AG156" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="157" spans="2:33" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Adiciona plano de furo Joao Canzi PV06 PV08
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DDC3DEE-9F23-4662-862F-278B02A0DDE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21062300-F63A-41E9-91D4-9236807A7D48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BASE_DASH_EXTENSAO" sheetId="1" r:id="rId1"/>
@@ -9057,7 +9057,7 @@
         <v>6</v>
       </c>
       <c r="F192" s="5">
-        <v>78.19</v>
+        <v>158.69999999999999</v>
       </c>
       <c r="L192" s="6"/>
       <c r="M192" s="6"/>
@@ -9073,7 +9073,8 @@
       <c r="W192" s="6"/>
       <c r="X192" s="6"/>
       <c r="Y192" s="6">
-        <v>78.19</v>
+        <f>78.19+80.53</f>
+        <v>158.72</v>
       </c>
       <c r="Z192" s="6"/>
       <c r="AA192" s="6"/>

</xml_diff>

<commit_message>
Atualiza PDS de maio e planilhas
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21062300-F63A-41E9-91D4-9236807A7D48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F5E3A9A-5019-4D99-8281-814FC022FA8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="121">
   <si>
     <t>Obra</t>
   </si>
@@ -9491,6 +9491,9 @@
       <c r="AD204" s="6"/>
       <c r="AE204" s="6"/>
       <c r="AF204" s="6"/>
+      <c r="AG204" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="205" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B205" t="s">
@@ -9526,6 +9529,9 @@
       <c r="AD205" s="6"/>
       <c r="AE205" s="6"/>
       <c r="AF205" s="6"/>
+      <c r="AG205" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="206" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B206" s="5" t="s">

</xml_diff>

<commit_message>
Atualiza bases e restaura Agua Vermelha MD
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F5E3A9A-5019-4D99-8281-814FC022FA8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCA6F4DA-0E96-4337-9D01-E8E0A6C3B1EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7272,7 +7272,7 @@
         <v>1799.2</v>
       </c>
       <c r="F145" s="5">
-        <v>9</v>
+        <v>81</v>
       </c>
       <c r="L145" s="6"/>
       <c r="M145" s="6"/>
@@ -7290,7 +7290,7 @@
       <c r="W145" s="6"/>
       <c r="X145" s="6"/>
       <c r="Y145" s="6">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="Z145" s="6"/>
       <c r="AA145" s="6"/>
@@ -7743,7 +7743,9 @@
       <c r="X157" s="6">
         <v>8.81</v>
       </c>
-      <c r="Y157" s="6"/>
+      <c r="Y157" s="6">
+        <v>70.84</v>
+      </c>
       <c r="Z157" s="6"/>
       <c r="AA157" s="6"/>
       <c r="AB157" s="6"/>
@@ -7752,7 +7754,7 @@
       <c r="AE157" s="6"/>
       <c r="AF157" s="6"/>
       <c r="AG157" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="158" spans="2:33" x14ac:dyDescent="0.3">
@@ -7810,7 +7812,7 @@
       <c r="AE158" s="6"/>
       <c r="AF158" s="6"/>
       <c r="AG158" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="159" spans="2:33" x14ac:dyDescent="0.3">
@@ -7844,7 +7846,10 @@
         <v>65.599999999999994</v>
       </c>
       <c r="X159" s="6"/>
-      <c r="Y159" s="6"/>
+      <c r="Y159" s="6">
+        <f>14.84+38.87+23.3</f>
+        <v>77.009999999999991</v>
+      </c>
       <c r="Z159" s="6"/>
       <c r="AA159" s="6"/>
       <c r="AB159" s="6"/>
@@ -7853,7 +7858,7 @@
       <c r="AE159" s="6"/>
       <c r="AF159" s="6"/>
       <c r="AG159" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="160" spans="2:33" x14ac:dyDescent="0.3">
@@ -7902,7 +7907,7 @@
       <c r="AE160" s="6"/>
       <c r="AF160" s="6"/>
       <c r="AG160" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="161" spans="2:33" x14ac:dyDescent="0.3">
@@ -7945,7 +7950,7 @@
       <c r="AE161" s="6"/>
       <c r="AF161" s="6"/>
       <c r="AG161" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="162" spans="2:33" x14ac:dyDescent="0.3">
@@ -8131,7 +8136,7 @@
       <c r="AE166" s="6"/>
       <c r="AF166" s="6"/>
       <c r="AG166" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="167" spans="2:33" x14ac:dyDescent="0.3">
@@ -8169,7 +8174,7 @@
       <c r="AE167" s="6"/>
       <c r="AF167" s="6"/>
       <c r="AG167" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="168" spans="2:33" x14ac:dyDescent="0.3">
@@ -8218,7 +8223,7 @@
       <c r="AE168" s="6"/>
       <c r="AF168" s="6"/>
       <c r="AG168" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="169" spans="2:33" x14ac:dyDescent="0.3">
@@ -8250,8 +8255,7 @@
       <c r="V169" s="6"/>
       <c r="W169" s="6"/>
       <c r="X169" s="6">
-        <f>11.35+17.44+12.11</f>
-        <v>40.9</v>
+        <v>47.56</v>
       </c>
       <c r="Y169" s="6"/>
       <c r="Z169" s="6"/>
@@ -8262,7 +8266,7 @@
       <c r="AE169" s="6"/>
       <c r="AF169" s="6"/>
       <c r="AG169" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="170" spans="2:33" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza planilhas do dashboard 2026-05-20
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3201084-D6CB-45F5-AA24-265FB3B68E58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CD3C055-8608-4998-951C-58DFEC9569E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3267,7 +3267,9 @@
       <c r="V52" s="6"/>
       <c r="W52" s="6"/>
       <c r="X52" s="6"/>
-      <c r="Y52" s="6"/>
+      <c r="Y52" s="6">
+        <v>84.32</v>
+      </c>
       <c r="Z52" s="6"/>
       <c r="AA52" s="6"/>
       <c r="AB52" s="6"/>
@@ -9061,7 +9063,7 @@
         <v>6</v>
       </c>
       <c r="F192" s="5">
-        <v>268.02</v>
+        <v>311.68</v>
       </c>
       <c r="L192" s="6"/>
       <c r="M192" s="6"/>
@@ -9077,7 +9079,7 @@
       <c r="W192" s="6"/>
       <c r="X192" s="6"/>
       <c r="Y192" s="6">
-        <v>268.02</v>
+        <v>311.68</v>
       </c>
       <c r="Z192" s="6"/>
       <c r="AA192" s="6"/>

</xml_diff>

<commit_message>
Atualiza base dash 2026-05-25
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8680C7E9-C780-447B-908C-14B9740642F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8266D4C-FEFC-4618-BE67-91F82CF17AD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9171,7 +9171,7 @@
         <v>34</v>
       </c>
       <c r="F195" s="3">
-        <v>374.4</v>
+        <v>454.5</v>
       </c>
       <c r="L195" s="4"/>
       <c r="M195" s="4"/>

</xml_diff>

<commit_message>
Atualiza base dash compatibilizada
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8266D4C-FEFC-4618-BE67-91F82CF17AD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF016727-AA40-4CC2-9C6F-750C3C0D77BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -817,17 +817,17 @@
     <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="produção Novembro 2025" dataDxfId="13"/>
     <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="produção Dezembro 2025" dataDxfId="12"/>
     <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="produção Janeiro 2026" dataDxfId="11"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="produção Fevereiro 2026" dataDxfId="10"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="produção Março 2026" dataDxfId="9"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="produção Abril 2026" dataDxfId="8"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="produção Maio 2026" dataDxfId="7"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="produção Junho 2026" dataDxfId="6"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="produção Julho 2026" dataDxfId="5"/>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="produção Agosto 2026" dataDxfId="4"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="produção Setembro 2026" dataDxfId="3"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="produção Outubro 2026" dataDxfId="2"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="produção Novembro 2026" dataDxfId="1"/>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="produção Dezembro 2026" dataDxfId="0"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="produção Fevereiro 2026" dataDxfId="0"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="produção Março 2026" dataDxfId="10"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="produção Abril 2026" dataDxfId="9"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="produção Maio 2026" dataDxfId="8"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="produção Junho 2026" dataDxfId="7"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="produção Julho 2026" dataDxfId="6"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="produção Agosto 2026" dataDxfId="5"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="produção Setembro 2026" dataDxfId="4"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="produção Outubro 2026" dataDxfId="3"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="produção Novembro 2026" dataDxfId="2"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="produção Dezembro 2026" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1118,7 +1118,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AG218"/>
+  <dimension ref="A1:AL218"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
@@ -1135,7 +1135,9 @@
     <col min="13" max="13" width="14" customWidth="1"/>
     <col min="14" max="15" width="7.6640625" customWidth="1"/>
     <col min="16" max="16" width="14.5546875" customWidth="1"/>
-    <col min="17" max="32" width="7.6640625" customWidth="1"/>
+    <col min="17" max="23" width="7.6640625" customWidth="1"/>
+    <col min="24" max="24" width="9.88671875" customWidth="1"/>
+    <col min="25" max="32" width="7.6640625" customWidth="1"/>
     <col min="33" max="33" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7251,7 +7253,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="145" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="145" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B145" t="s">
         <v>67</v>
       </c>
@@ -7289,7 +7291,7 @@
       <c r="AE145" s="4"/>
       <c r="AF145" s="4"/>
     </row>
-    <row r="146" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="146" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B146" t="s">
         <v>67</v>
       </c>
@@ -7324,7 +7326,7 @@
       <c r="AE146" s="4"/>
       <c r="AF146" s="4"/>
     </row>
-    <row r="147" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="147" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B147" t="s">
         <v>68</v>
       </c>
@@ -7359,7 +7361,7 @@
       <c r="AE147" s="4"/>
       <c r="AF147" s="4"/>
     </row>
-    <row r="148" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="148" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B148" t="s">
         <v>68</v>
       </c>
@@ -7394,7 +7396,7 @@
       <c r="AE148" s="4"/>
       <c r="AF148" s="4"/>
     </row>
-    <row r="149" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="149" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B149" t="s">
         <v>69</v>
       </c>
@@ -7435,7 +7437,7 @@
       <c r="AE149" s="4"/>
       <c r="AF149" s="4"/>
     </row>
-    <row r="150" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="150" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B150" t="s">
         <v>69</v>
       </c>
@@ -7480,7 +7482,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="151" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="151" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B151" t="s">
         <v>70</v>
       </c>
@@ -7512,7 +7514,7 @@
       <c r="AE151" s="4"/>
       <c r="AF151" s="4"/>
     </row>
-    <row r="152" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="152" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B152" t="s">
         <v>70</v>
       </c>
@@ -7547,7 +7549,7 @@
       <c r="AE152" s="4"/>
       <c r="AF152" s="4"/>
     </row>
-    <row r="153" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="153" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B153" t="s">
         <v>71</v>
       </c>
@@ -7582,7 +7584,7 @@
       <c r="AE153" s="4"/>
       <c r="AF153" s="4"/>
     </row>
-    <row r="154" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="154" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B154" t="s">
         <v>71</v>
       </c>
@@ -7617,7 +7619,7 @@
       <c r="AE154" s="4"/>
       <c r="AF154" s="4"/>
     </row>
-    <row r="155" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="155" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B155" t="s">
         <v>72</v>
       </c>
@@ -7651,8 +7653,11 @@
       <c r="AD155" s="4"/>
       <c r="AE155" s="4"/>
       <c r="AF155" s="4"/>
-    </row>
-    <row r="156" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AL155">
+        <v>1746.61</v>
+      </c>
+    </row>
+    <row r="156" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B156" t="s">
         <v>72</v>
       </c>
@@ -7686,8 +7691,11 @@
       <c r="AD156" s="4"/>
       <c r="AE156" s="4"/>
       <c r="AF156" s="4"/>
-    </row>
-    <row r="157" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AL156">
+        <v>1471.49</v>
+      </c>
+    </row>
+    <row r="157" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B157" t="s">
         <v>73</v>
       </c>
@@ -7724,8 +7732,12 @@
       <c r="AG157" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="158" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AL157">
+        <f>AL155-AL156</f>
+        <v>275.11999999999989</v>
+      </c>
+    </row>
+    <row r="158" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B158" t="s">
         <v>73</v>
       </c>
@@ -7763,7 +7775,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="159" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="159" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B159" s="3" t="s">
         <v>75</v>
       </c>
@@ -7777,7 +7789,7 @@
         <v>240.4</v>
       </c>
       <c r="F159" s="3">
-        <v>582.63</v>
+        <v>766.04399999999998</v>
       </c>
       <c r="G159">
         <v>18</v>
@@ -7801,12 +7813,12 @@
       <c r="S159" s="4"/>
       <c r="T159" s="4"/>
       <c r="U159" s="4">
-        <f>528.5-68.36</f>
-        <v>460.14</v>
+        <f>528.5-68.36+91.707</f>
+        <v>551.84699999999998</v>
       </c>
       <c r="V159" s="4">
-        <f>52.4-0.15</f>
-        <v>52.25</v>
+        <f>52.4-0.15+91.707</f>
+        <v>143.95699999999999</v>
       </c>
       <c r="W159" s="4"/>
       <c r="X159" s="4">
@@ -7824,7 +7836,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="160" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="160" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B160" s="3" t="s">
         <v>75</v>
       </c>
@@ -7872,6 +7884,10 @@
       <c r="AG160" t="s">
         <v>74</v>
       </c>
+      <c r="AL160">
+        <f>AL157/3</f>
+        <v>91.706666666666635</v>
+      </c>
     </row>
     <row r="161" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B161" s="3" t="s">
@@ -7887,7 +7903,7 @@
         <v>286</v>
       </c>
       <c r="F161" s="3">
-        <v>374.7</v>
+        <v>466.40699999999998</v>
       </c>
       <c r="G161">
         <v>8</v>
@@ -7915,7 +7931,8 @@
         <v>118.2</v>
       </c>
       <c r="V161" s="4">
-        <v>256.5</v>
+        <f>256.5+91.707</f>
+        <v>348.20699999999999</v>
       </c>
       <c r="W161" s="4"/>
       <c r="X161" s="4"/>

</xml_diff>

<commit_message>
Atualiza PDS e mapa 2026-05-26
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF016727-AA40-4CC2-9C6F-750C3C0D77BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5CE51A2-4BD7-44B5-B94A-3CAAE165E5C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="645" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="125">
   <si>
     <t>Data</t>
   </si>
@@ -817,17 +817,17 @@
     <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="produção Novembro 2025" dataDxfId="13"/>
     <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="produção Dezembro 2025" dataDxfId="12"/>
     <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="produção Janeiro 2026" dataDxfId="11"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="produção Fevereiro 2026" dataDxfId="0"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="produção Março 2026" dataDxfId="10"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="produção Abril 2026" dataDxfId="9"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="produção Maio 2026" dataDxfId="8"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="produção Junho 2026" dataDxfId="7"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="produção Julho 2026" dataDxfId="6"/>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="produção Agosto 2026" dataDxfId="5"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="produção Setembro 2026" dataDxfId="4"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="produção Outubro 2026" dataDxfId="3"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="produção Novembro 2026" dataDxfId="2"/>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="produção Dezembro 2026" dataDxfId="1"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="produção Fevereiro 2026" dataDxfId="10"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="produção Março 2026" dataDxfId="9"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="produção Abril 2026" dataDxfId="8"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="produção Maio 2026" dataDxfId="7"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="produção Junho 2026" dataDxfId="6"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="produção Julho 2026" dataDxfId="5"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="produção Agosto 2026" dataDxfId="4"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="produção Setembro 2026" dataDxfId="3"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="produção Outubro 2026" dataDxfId="2"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="produção Novembro 2026" dataDxfId="1"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="produção Dezembro 2026" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3304,7 +3304,7 @@
         <v>0</v>
       </c>
       <c r="F54">
-        <v>84.32</v>
+        <v>162.9</v>
       </c>
       <c r="K54" s="2"/>
       <c r="L54" s="4"/>
@@ -3321,7 +3321,8 @@
       <c r="W54" s="4"/>
       <c r="X54" s="4"/>
       <c r="Y54" s="4">
-        <v>84.32</v>
+        <f>78.58+84.32</f>
+        <v>162.89999999999998</v>
       </c>
       <c r="Z54" s="4"/>
       <c r="AA54" s="4"/>
@@ -8039,6 +8040,9 @@
       <c r="AD163" s="4"/>
       <c r="AE163" s="4"/>
       <c r="AF163" s="4"/>
+      <c r="AG163" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="164" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B164" s="3" t="s">
@@ -8079,6 +8083,9 @@
       <c r="AD164" s="4"/>
       <c r="AE164" s="4"/>
       <c r="AF164" s="4"/>
+      <c r="AG164" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="165" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B165" t="s">

</xml_diff>

<commit_message>
Atualiza planilhas EAP e dashboard
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5CE51A2-4BD7-44B5-B94A-3CAAE165E5C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{025F1614-BF82-4C33-923E-358A18CE3888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7452,7 +7452,7 @@
         <v>1799.2</v>
       </c>
       <c r="F150" s="3">
-        <v>81</v>
+        <v>282</v>
       </c>
       <c r="L150" s="4"/>
       <c r="M150" s="4"/>
@@ -7470,7 +7470,7 @@
       <c r="W150" s="4"/>
       <c r="X150" s="4"/>
       <c r="Y150" s="4">
-        <v>72</v>
+        <v>273</v>
       </c>
       <c r="Z150" s="4"/>
       <c r="AA150" s="4"/>

</xml_diff>

<commit_message>
Corrige Base Dash Sao Lucas 273m
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{025F1614-BF82-4C33-923E-358A18CE3888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39D15A9C-A368-465C-860A-542118E352C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7452,7 +7452,7 @@
         <v>1799.2</v>
       </c>
       <c r="F150" s="3">
-        <v>282</v>
+        <v>273</v>
       </c>
       <c r="L150" s="4"/>
       <c r="M150" s="4"/>

</xml_diff>

<commit_message>
Atualiza PDS e plano de furo Lourdes
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B86F1CA1-20F9-4B5A-89D3-47DC3706369A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE0B521B-21D3-4A64-8CFA-71029D5E5BDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BASE_DASH_EXTENSAO" sheetId="1" r:id="rId1"/>
@@ -3304,7 +3304,7 @@
         <v>0</v>
       </c>
       <c r="F54">
-        <v>162.9</v>
+        <v>308.3</v>
       </c>
       <c r="K54" s="2"/>
       <c r="L54" s="4"/>
@@ -3321,8 +3321,8 @@
       <c r="W54" s="4"/>
       <c r="X54" s="4"/>
       <c r="Y54" s="4">
-        <f>78.58+84.32</f>
-        <v>162.89999999999998</v>
+        <f>78.58+84.32+66.57+78.843</f>
+        <v>308.31299999999999</v>
       </c>
       <c r="Z54" s="4"/>
       <c r="AA54" s="4"/>

</xml_diff>

<commit_message>
Atualiza planilhas EAP e base dash
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE0B521B-21D3-4A64-8CFA-71029D5E5BDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{196EAB5F-F9DC-44BF-86A5-A2D3BA47891F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="125">
   <si>
     <t>Data</t>
   </si>
@@ -8805,6 +8805,9 @@
       <c r="AD183" s="4"/>
       <c r="AE183" s="4"/>
       <c r="AF183" s="4"/>
+      <c r="AG183" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="184" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B184" t="s">
@@ -9193,7 +9196,7 @@
         <v>34</v>
       </c>
       <c r="F195" s="3">
-        <v>592.20000000000005</v>
+        <v>454.56</v>
       </c>
       <c r="L195" s="4"/>
       <c r="M195" s="4"/>
@@ -9209,8 +9212,7 @@
       <c r="W195" s="4"/>
       <c r="X195" s="4"/>
       <c r="Y195" s="4">
-        <f>62.701+311.68+80.157+52.62+85.03</f>
-        <v>592.18799999999999</v>
+        <v>454.56</v>
       </c>
       <c r="Z195" s="4"/>
       <c r="AA195" s="4"/>

</xml_diff>

<commit_message>
Atualiza seguranca e mapa Joao Canzi
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{196EAB5F-F9DC-44BF-86A5-A2D3BA47891F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F631A82-82E5-4D48-97A4-6D3A1211F86F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BASE_DASH_EXTENSAO" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="125">
   <si>
     <t>Data</t>
   </si>
@@ -3247,9 +3247,6 @@
       <c r="AD52" s="4"/>
       <c r="AE52" s="4"/>
       <c r="AF52" s="4"/>
-      <c r="AG52" t="s">
-        <v>40</v>
-      </c>
     </row>
     <row r="53" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B53" t="s">
@@ -3286,9 +3283,6 @@
       <c r="AD53" s="4"/>
       <c r="AE53" s="4"/>
       <c r="AF53" s="4"/>
-      <c r="AG53" t="s">
-        <v>35</v>
-      </c>
     </row>
     <row r="54" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B54" s="3" t="s">
@@ -3303,7 +3297,7 @@
       <c r="E54">
         <v>0</v>
       </c>
-      <c r="F54">
+      <c r="F54" s="3">
         <v>308.3</v>
       </c>
       <c r="K54" s="2"/>
@@ -3332,7 +3326,7 @@
       <c r="AE54" s="4"/>
       <c r="AF54" s="4"/>
       <c r="AG54" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="55" spans="2:33" x14ac:dyDescent="0.3">
@@ -7452,7 +7446,7 @@
         <v>1799.2</v>
       </c>
       <c r="F150" s="3">
-        <v>345</v>
+        <v>888</v>
       </c>
       <c r="L150" s="4"/>
       <c r="M150" s="4"/>
@@ -7468,7 +7462,7 @@
       <c r="W150" s="4"/>
       <c r="X150" s="4"/>
       <c r="Y150" s="4">
-        <v>345</v>
+        <v>888</v>
       </c>
       <c r="Z150" s="4"/>
       <c r="AA150" s="4"/>
@@ -7728,9 +7722,6 @@
       <c r="AD157" s="4"/>
       <c r="AE157" s="4"/>
       <c r="AF157" s="4"/>
-      <c r="AG157" t="s">
-        <v>74</v>
-      </c>
       <c r="AL157">
         <f>AL155-AL156</f>
         <v>275.11999999999989</v>
@@ -7770,9 +7761,6 @@
       <c r="AD158" s="4"/>
       <c r="AE158" s="4"/>
       <c r="AF158" s="4"/>
-      <c r="AG158" t="s">
-        <v>74</v>
-      </c>
     </row>
     <row r="159" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B159" s="3" t="s">
@@ -8680,9 +8668,6 @@
       <c r="AD180" s="4"/>
       <c r="AE180" s="4"/>
       <c r="AF180" s="4"/>
-      <c r="AG180" t="s">
-        <v>35</v>
-      </c>
     </row>
     <row r="181" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B181" s="3" t="s">
@@ -8773,6 +8758,9 @@
       <c r="AD182" s="4"/>
       <c r="AE182" s="4"/>
       <c r="AF182" s="4"/>
+      <c r="AG182" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="183" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B183" t="s">
@@ -9196,7 +9184,7 @@
         <v>34</v>
       </c>
       <c r="F195" s="3">
-        <v>454.56</v>
+        <v>539.59</v>
       </c>
       <c r="L195" s="4"/>
       <c r="M195" s="4"/>
@@ -9212,7 +9200,8 @@
       <c r="W195" s="4"/>
       <c r="X195" s="4"/>
       <c r="Y195" s="4">
-        <v>454.56</v>
+        <f>454.56+85.03</f>
+        <v>539.59</v>
       </c>
       <c r="Z195" s="4"/>
       <c r="AA195" s="4"/>
@@ -9668,7 +9657,9 @@
       <c r="V208" s="4"/>
       <c r="W208" s="4"/>
       <c r="X208" s="4"/>
-      <c r="Y208" s="4"/>
+      <c r="Y208" s="4">
+        <v>56.1</v>
+      </c>
       <c r="Z208" s="4"/>
       <c r="AA208" s="4"/>
       <c r="AB208" s="4"/>
@@ -10061,9 +10052,9 @@
   </sheetData>
   <autoFilter ref="A1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Atualiza PDS e mapa Joao Canzi PV14 PV15
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F631A82-82E5-4D48-97A4-6D3A1211F86F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17A871C8-6823-4757-B691-A06C4DCFF530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BASE_DASH_EXTENSAO" sheetId="1" r:id="rId1"/>
@@ -9644,6 +9644,9 @@
       <c r="E208">
         <v>95</v>
       </c>
+      <c r="F208" s="3">
+        <v>56.1</v>
+      </c>
       <c r="L208" s="4"/>
       <c r="M208" s="4"/>
       <c r="N208" s="4"/>

</xml_diff>

<commit_message>
Atualiza PDS, planilhas e planos de furo
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A69902AD-2067-401B-909F-C333BE192426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EA2308F-CEEB-4798-A0F0-6CF4B79DAA64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25245" yWindow="4230" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BASE_DASH_EXTENSAO" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="125">
   <si>
     <t>Data</t>
   </si>
@@ -2568,8 +2568,11 @@
       <c r="AD32" s="4"/>
       <c r="AE32" s="4"/>
       <c r="AF32" s="4"/>
-    </row>
-    <row r="33" spans="2:32" x14ac:dyDescent="0.3">
+      <c r="AG32" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="33" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
         <v>44</v>
       </c>
@@ -2603,8 +2606,11 @@
       <c r="AD33" s="4"/>
       <c r="AE33" s="4"/>
       <c r="AF33" s="4"/>
-    </row>
-    <row r="34" spans="2:32" x14ac:dyDescent="0.3">
+      <c r="AG33" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="34" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B34" t="s">
         <v>45</v>
       </c>
@@ -2636,7 +2642,7 @@
       <c r="AE34" s="4"/>
       <c r="AF34" s="4"/>
     </row>
-    <row r="35" spans="2:32" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
         <v>45</v>
       </c>
@@ -2671,7 +2677,7 @@
       <c r="AE35" s="4"/>
       <c r="AF35" s="4"/>
     </row>
-    <row r="36" spans="2:32" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
         <v>46</v>
       </c>
@@ -2703,7 +2709,7 @@
       <c r="AE36" s="4"/>
       <c r="AF36" s="4"/>
     </row>
-    <row r="37" spans="2:32" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
         <v>46</v>
       </c>
@@ -2738,7 +2744,7 @@
       <c r="AE37" s="4"/>
       <c r="AF37" s="4"/>
     </row>
-    <row r="38" spans="2:32" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
         <v>47</v>
       </c>
@@ -2769,8 +2775,11 @@
       <c r="AD38" s="4"/>
       <c r="AE38" s="4"/>
       <c r="AF38" s="4"/>
-    </row>
-    <row r="39" spans="2:32" x14ac:dyDescent="0.3">
+      <c r="AG38" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="39" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B39" t="s">
         <v>47</v>
       </c>
@@ -2805,7 +2814,7 @@
       <c r="AE39" s="4"/>
       <c r="AF39" s="4"/>
     </row>
-    <row r="40" spans="2:32" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
         <v>48</v>
       </c>
@@ -2840,7 +2849,7 @@
       <c r="AE40" s="4"/>
       <c r="AF40" s="4"/>
     </row>
-    <row r="41" spans="2:32" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B41" t="s">
         <v>48</v>
       </c>
@@ -2872,7 +2881,7 @@
       <c r="AE41" s="4"/>
       <c r="AF41" s="4"/>
     </row>
-    <row r="42" spans="2:32" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
         <v>49</v>
       </c>
@@ -2907,7 +2916,7 @@
       <c r="AE42" s="4"/>
       <c r="AF42" s="4"/>
     </row>
-    <row r="43" spans="2:32" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B43" t="s">
         <v>49</v>
       </c>
@@ -2939,7 +2948,7 @@
       <c r="AE43" s="4"/>
       <c r="AF43" s="4"/>
     </row>
-    <row r="44" spans="2:32" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B44" t="s">
         <v>50</v>
       </c>
@@ -2974,7 +2983,7 @@
       <c r="AE44" s="4"/>
       <c r="AF44" s="4"/>
     </row>
-    <row r="45" spans="2:32" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B45" t="s">
         <v>50</v>
       </c>
@@ -3006,7 +3015,7 @@
       <c r="AE45" s="4"/>
       <c r="AF45" s="4"/>
     </row>
-    <row r="46" spans="2:32" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B46" t="s">
         <v>51</v>
       </c>
@@ -3041,7 +3050,7 @@
       <c r="AE46" s="4"/>
       <c r="AF46" s="4"/>
     </row>
-    <row r="47" spans="2:32" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B47" t="s">
         <v>51</v>
       </c>
@@ -3076,7 +3085,7 @@
       <c r="AE47" s="4"/>
       <c r="AF47" s="4"/>
     </row>
-    <row r="48" spans="2:32" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B48" t="s">
         <v>52</v>
       </c>
@@ -7446,7 +7455,7 @@
         <v>1799.2</v>
       </c>
       <c r="F150" s="3">
-        <v>888</v>
+        <v>943.4</v>
       </c>
       <c r="L150" s="4"/>
       <c r="M150" s="4"/>
@@ -7464,7 +7473,9 @@
       <c r="Y150" s="4">
         <v>888</v>
       </c>
-      <c r="Z150" s="4"/>
+      <c r="Z150" s="4">
+        <v>55.4</v>
+      </c>
       <c r="AA150" s="4"/>
       <c r="AB150" s="4"/>
       <c r="AC150" s="4"/>
@@ -8936,6 +8947,9 @@
       <c r="AD187" s="4"/>
       <c r="AE187" s="4"/>
       <c r="AF187" s="4"/>
+      <c r="AG187" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="188" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B188" t="s">
@@ -8971,6 +8985,9 @@
       <c r="AD188" s="4"/>
       <c r="AE188" s="4"/>
       <c r="AF188" s="4"/>
+      <c r="AG188" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="189" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B189" t="s">
@@ -9184,7 +9201,7 @@
         <v>34</v>
       </c>
       <c r="F195" s="3">
-        <v>592.21</v>
+        <v>736.35</v>
       </c>
       <c r="L195" s="4"/>
       <c r="M195" s="4"/>
@@ -9202,7 +9219,10 @@
       <c r="Y195" s="4">
         <v>592.21</v>
       </c>
-      <c r="Z195" s="4"/>
+      <c r="Z195" s="4">
+        <f>64.57+79.57</f>
+        <v>144.13999999999999</v>
+      </c>
       <c r="AA195" s="4"/>
       <c r="AB195" s="4"/>
       <c r="AC195" s="4"/>
@@ -9355,6 +9375,9 @@
       <c r="AD199" s="4"/>
       <c r="AE199" s="4"/>
       <c r="AF199" s="4"/>
+      <c r="AG199" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="200" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B200" t="s">
@@ -9390,6 +9413,9 @@
       <c r="AD200" s="4"/>
       <c r="AE200" s="4"/>
       <c r="AF200" s="4"/>
+      <c r="AG200" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="201" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B201" t="s">
@@ -9644,7 +9670,7 @@
         <v>95</v>
       </c>
       <c r="F208" s="3">
-        <v>56.1</v>
+        <v>93.1</v>
       </c>
       <c r="L208" s="4"/>
       <c r="M208" s="4"/>
@@ -9662,7 +9688,9 @@
       <c r="Y208" s="4">
         <v>56.1</v>
       </c>
-      <c r="Z208" s="4"/>
+      <c r="Z208" s="4">
+        <v>37</v>
+      </c>
       <c r="AA208" s="4"/>
       <c r="AB208" s="4"/>
       <c r="AC208" s="4"/>

</xml_diff>

<commit_message>
Atualiza PDS e mapa 2026-06-09
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EA2308F-CEEB-4798-A0F0-6CF4B79DAA64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{169ADDE0-D6CC-47F5-BD01-014BA377EE8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8978,7 +8978,9 @@
       <c r="W188" s="4"/>
       <c r="X188" s="4"/>
       <c r="Y188" s="4"/>
-      <c r="Z188" s="4"/>
+      <c r="Z188" s="4">
+        <v>103.03</v>
+      </c>
       <c r="AA188" s="4"/>
       <c r="AB188" s="4"/>
       <c r="AC188" s="4"/>
@@ -9220,8 +9222,8 @@
         <v>592.21</v>
       </c>
       <c r="Z195" s="4">
-        <f>64.57+79.57</f>
-        <v>144.13999999999999</v>
+        <f>64.57+79.57+66.725</f>
+        <v>210.86499999999998</v>
       </c>
       <c r="AA195" s="4"/>
       <c r="AB195" s="4"/>
@@ -9406,7 +9408,9 @@
       <c r="W200" s="4"/>
       <c r="X200" s="4"/>
       <c r="Y200" s="4"/>
-      <c r="Z200" s="4"/>
+      <c r="Z200" s="4">
+        <v>20.2</v>
+      </c>
       <c r="AA200" s="4"/>
       <c r="AB200" s="4"/>
       <c r="AC200" s="4"/>

</xml_diff>

<commit_message>
Atualiza executado da base dash
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{169ADDE0-D6CC-47F5-BD01-014BA377EE8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{206CF054-EACD-405E-B087-782B00BED439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8964,6 +8964,9 @@
       <c r="E188">
         <v>338.5</v>
       </c>
+      <c r="F188" s="3">
+        <v>103.03</v>
+      </c>
       <c r="L188" s="4"/>
       <c r="M188" s="4"/>
       <c r="N188" s="4"/>
@@ -9203,7 +9206,7 @@
         <v>34</v>
       </c>
       <c r="F195" s="3">
-        <v>736.35</v>
+        <v>759.41499999999996</v>
       </c>
       <c r="L195" s="4"/>
       <c r="M195" s="4"/>
@@ -9219,7 +9222,8 @@
       <c r="W195" s="4"/>
       <c r="X195" s="4"/>
       <c r="Y195" s="4">
-        <v>592.21</v>
+        <f>592.21-43.66</f>
+        <v>548.55000000000007</v>
       </c>
       <c r="Z195" s="4">
         <f>64.57+79.57+66.725</f>
@@ -9394,6 +9398,9 @@
       <c r="E200">
         <v>180</v>
       </c>
+      <c r="F200" s="3">
+        <v>63.86</v>
+      </c>
       <c r="L200" s="4"/>
       <c r="M200" s="4"/>
       <c r="N200" s="4"/>
@@ -9407,7 +9414,9 @@
       <c r="V200" s="4"/>
       <c r="W200" s="4"/>
       <c r="X200" s="4"/>
-      <c r="Y200" s="4"/>
+      <c r="Y200" s="4">
+        <v>43.66</v>
+      </c>
       <c r="Z200" s="4">
         <v>20.2</v>
       </c>

</xml_diff>

<commit_message>
Atualiza PDS e planilhas 2026-06-22
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FEB0680-7D73-42CE-B2B5-65BD18FBBC34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECE93373-2C15-4A62-A2D8-97CA376E985F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BASE_DASH_EXTENSAO" sheetId="1" r:id="rId1"/>
@@ -2807,7 +2807,9 @@
       <c r="W39" s="4"/>
       <c r="X39" s="4"/>
       <c r="Y39" s="4"/>
-      <c r="Z39" s="4"/>
+      <c r="Z39" s="4">
+        <v>11.5</v>
+      </c>
       <c r="AA39" s="4"/>
       <c r="AB39" s="4"/>
       <c r="AC39" s="4"/>
@@ -7475,7 +7477,7 @@
         <v>888</v>
       </c>
       <c r="Z150" s="4">
-        <v>339.2</v>
+        <v>428.7</v>
       </c>
       <c r="AA150" s="4"/>
       <c r="AB150" s="4"/>
@@ -8836,7 +8838,9 @@
       <c r="W184" s="4"/>
       <c r="X184" s="4"/>
       <c r="Y184" s="4"/>
-      <c r="Z184" s="4"/>
+      <c r="Z184" s="4">
+        <v>42</v>
+      </c>
       <c r="AA184" s="4"/>
       <c r="AB184" s="4"/>
       <c r="AC184" s="4"/>
@@ -9419,7 +9423,7 @@
         <v>43.66</v>
       </c>
       <c r="Z200" s="4">
-        <v>25.2</v>
+        <v>117.2</v>
       </c>
       <c r="AA200" s="4"/>
       <c r="AB200" s="4"/>

</xml_diff>

<commit_message>
Atualiza planilhas e corrige custos de funcionarios
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77884FDC-C6A3-407C-BDD4-AF07C4518E02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB2EF3D5-C9E1-4C09-AF92-C9E53AEC36D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="125">
   <si>
     <t>Data</t>
   </si>
@@ -7464,7 +7464,7 @@
         <v>1799.2</v>
       </c>
       <c r="F150" s="3">
-        <v>1316.7</v>
+        <v>1403.2</v>
       </c>
       <c r="L150" s="4"/>
       <c r="M150" s="4"/>
@@ -7483,7 +7483,7 @@
         <v>888</v>
       </c>
       <c r="Z150" s="4">
-        <v>428.7</v>
+        <v>515.20000000000005</v>
       </c>
       <c r="AA150" s="4"/>
       <c r="AB150" s="4"/>
@@ -9591,6 +9591,9 @@
       <c r="D205" t="s">
         <v>34</v>
       </c>
+      <c r="F205" s="3">
+        <v>24</v>
+      </c>
       <c r="L205" s="4"/>
       <c r="M205" s="4"/>
       <c r="N205" s="4"/>
@@ -9605,13 +9608,18 @@
       <c r="W205" s="4"/>
       <c r="X205" s="4"/>
       <c r="Y205" s="4"/>
-      <c r="Z205" s="4"/>
+      <c r="Z205" s="4">
+        <v>24</v>
+      </c>
       <c r="AA205" s="4"/>
       <c r="AB205" s="4"/>
       <c r="AC205" s="4"/>
       <c r="AD205" s="4"/>
       <c r="AE205" s="4"/>
       <c r="AF205" s="4"/>
+      <c r="AG205" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="206" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B206" t="s">

</xml_diff>

<commit_message>
Atualizar bases de extensao EAP e seguranca
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB2EF3D5-C9E1-4C09-AF92-C9E53AEC36D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA516CB1-52F3-42DF-A693-8663F4E35CFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="126">
   <si>
     <t>Data</t>
   </si>
@@ -412,6 +412,9 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t xml:space="preserve">rede existente </t>
   </si>
 </sst>
 </file>
@@ -792,7 +795,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tb_base_dash_extensao" displayName="tb_base_dash_extensao" ref="B1:AF218">
-  <autoFilter ref="B1:AF218" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <autoFilter ref="B1:AF218" xr:uid="{00000000-0009-0000-0100-000001000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="RCE RUA JOSÉ MILITÃO"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="31">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Obra"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Bloco"/>
@@ -1133,7 +1142,7 @@
     <col min="14" max="15" width="7.6640625" customWidth="1"/>
     <col min="16" max="16" width="14.5546875" customWidth="1"/>
     <col min="17" max="21" width="7.6640625" customWidth="1"/>
-    <col min="22" max="22" width="36" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="20.33203125" customWidth="1"/>
     <col min="23" max="23" width="7.6640625" customWidth="1"/>
     <col min="24" max="24" width="9.88671875" customWidth="1"/>
     <col min="25" max="32" width="7.6640625" customWidth="1"/>
@@ -1241,7 +1250,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B2" s="3" t="s">
         <v>33</v>
       </c>
@@ -1287,7 +1296,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B3" s="3" t="s">
         <v>33</v>
       </c>
@@ -1330,7 +1339,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>33</v>
       </c>
@@ -1375,7 +1384,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B5" s="3" t="s">
         <v>33</v>
       </c>
@@ -1418,7 +1427,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
         <v>33</v>
       </c>
@@ -1461,7 +1470,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B7" s="3" t="s">
         <v>33</v>
       </c>
@@ -1504,7 +1513,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B8" s="3" t="s">
         <v>33</v>
       </c>
@@ -1552,7 +1561,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B9" s="3" t="s">
         <v>33</v>
       </c>
@@ -1596,7 +1605,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B10" s="3" t="s">
         <v>37</v>
       </c>
@@ -1653,7 +1662,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B11" s="3" t="s">
         <v>37</v>
       </c>
@@ -1691,7 +1700,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B12" s="3" t="s">
         <v>37</v>
       </c>
@@ -1742,7 +1751,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B13" s="3" t="s">
         <v>37</v>
       </c>
@@ -1783,7 +1792,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
         <v>37</v>
       </c>
@@ -1834,7 +1843,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B15" s="3" t="s">
         <v>37</v>
       </c>
@@ -1877,7 +1886,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
         <v>37</v>
       </c>
@@ -1930,7 +1939,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B17" s="3" t="s">
         <v>37</v>
       </c>
@@ -1968,7 +1977,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="18" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B18" s="3" t="s">
         <v>37</v>
       </c>
@@ -2017,7 +2026,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B19" s="3" t="s">
         <v>37</v>
       </c>
@@ -2066,7 +2075,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B20" s="3" t="s">
         <v>38</v>
       </c>
@@ -2121,7 +2130,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="21" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B21" s="3" t="s">
         <v>38</v>
       </c>
@@ -2164,7 +2173,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B22" s="3" t="s">
         <v>38</v>
       </c>
@@ -2213,7 +2222,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B23" s="3" t="s">
         <v>38</v>
       </c>
@@ -2256,7 +2265,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="24" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>39</v>
       </c>
@@ -2297,7 +2306,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="25" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>39</v>
       </c>
@@ -2332,7 +2341,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="26" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>41</v>
       </c>
@@ -2367,7 +2376,7 @@
       <c r="AE26" s="4"/>
       <c r="AF26" s="4"/>
     </row>
-    <row r="27" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>41</v>
       </c>
@@ -2402,7 +2411,7 @@
       <c r="AE27" s="4"/>
       <c r="AF27" s="4"/>
     </row>
-    <row r="28" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>42</v>
       </c>
@@ -2437,7 +2446,7 @@
       <c r="AE28" s="4"/>
       <c r="AF28" s="4"/>
     </row>
-    <row r="29" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B29" t="s">
         <v>42</v>
       </c>
@@ -2469,7 +2478,7 @@
       <c r="AE29" s="4"/>
       <c r="AF29" s="4"/>
     </row>
-    <row r="30" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
         <v>43</v>
       </c>
@@ -2501,7 +2510,7 @@
       <c r="AE30" s="4"/>
       <c r="AF30" s="4"/>
     </row>
-    <row r="31" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
         <v>43</v>
       </c>
@@ -2536,7 +2545,7 @@
       <c r="AE31" s="4"/>
       <c r="AF31" s="4"/>
     </row>
-    <row r="32" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
         <v>44</v>
       </c>
@@ -2576,7 +2585,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="33" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
         <v>44</v>
       </c>
@@ -2614,7 +2623,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="34" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B34" t="s">
         <v>45</v>
       </c>
@@ -2646,7 +2655,7 @@
       <c r="AE34" s="4"/>
       <c r="AF34" s="4"/>
     </row>
-    <row r="35" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
         <v>45</v>
       </c>
@@ -2681,7 +2690,7 @@
       <c r="AE35" s="4"/>
       <c r="AF35" s="4"/>
     </row>
-    <row r="36" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
         <v>46</v>
       </c>
@@ -2713,7 +2722,7 @@
       <c r="AE36" s="4"/>
       <c r="AF36" s="4"/>
     </row>
-    <row r="37" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
         <v>46</v>
       </c>
@@ -2748,7 +2757,7 @@
       <c r="AE37" s="4"/>
       <c r="AF37" s="4"/>
     </row>
-    <row r="38" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
         <v>47</v>
       </c>
@@ -2783,7 +2792,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="39" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B39" t="s">
         <v>47</v>
       </c>
@@ -2823,7 +2832,7 @@
       <c r="AE39" s="4"/>
       <c r="AF39" s="4"/>
     </row>
-    <row r="40" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
         <v>48</v>
       </c>
@@ -2858,7 +2867,7 @@
       <c r="AE40" s="4"/>
       <c r="AF40" s="4"/>
     </row>
-    <row r="41" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B41" t="s">
         <v>48</v>
       </c>
@@ -2890,7 +2899,7 @@
       <c r="AE41" s="4"/>
       <c r="AF41" s="4"/>
     </row>
-    <row r="42" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
         <v>49</v>
       </c>
@@ -2925,7 +2934,7 @@
       <c r="AE42" s="4"/>
       <c r="AF42" s="4"/>
     </row>
-    <row r="43" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B43" t="s">
         <v>49</v>
       </c>
@@ -2957,7 +2966,7 @@
       <c r="AE43" s="4"/>
       <c r="AF43" s="4"/>
     </row>
-    <row r="44" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B44" t="s">
         <v>50</v>
       </c>
@@ -2992,7 +3001,7 @@
       <c r="AE44" s="4"/>
       <c r="AF44" s="4"/>
     </row>
-    <row r="45" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B45" t="s">
         <v>50</v>
       </c>
@@ -3024,7 +3033,7 @@
       <c r="AE45" s="4"/>
       <c r="AF45" s="4"/>
     </row>
-    <row r="46" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B46" t="s">
         <v>51</v>
       </c>
@@ -3059,7 +3068,7 @@
       <c r="AE46" s="4"/>
       <c r="AF46" s="4"/>
     </row>
-    <row r="47" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B47" t="s">
         <v>51</v>
       </c>
@@ -3094,7 +3103,7 @@
       <c r="AE47" s="4"/>
       <c r="AF47" s="4"/>
     </row>
-    <row r="48" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B48" t="s">
         <v>52</v>
       </c>
@@ -3129,7 +3138,7 @@
       <c r="AE48" s="4"/>
       <c r="AF48" s="4"/>
     </row>
-    <row r="49" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B49" t="s">
         <v>52</v>
       </c>
@@ -3164,7 +3173,7 @@
       <c r="AE49" s="4"/>
       <c r="AF49" s="4"/>
     </row>
-    <row r="50" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B50" t="s">
         <v>53</v>
       </c>
@@ -3199,7 +3208,7 @@
       <c r="AE50" s="4"/>
       <c r="AF50" s="4"/>
     </row>
-    <row r="51" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B51" t="s">
         <v>53</v>
       </c>
@@ -3234,7 +3243,7 @@
       <c r="AE51" s="4"/>
       <c r="AF51" s="4"/>
     </row>
-    <row r="52" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B52" t="s">
         <v>54</v>
       </c>
@@ -3266,7 +3275,7 @@
       <c r="AE52" s="4"/>
       <c r="AF52" s="4"/>
     </row>
-    <row r="53" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B53" t="s">
         <v>54</v>
       </c>
@@ -3302,7 +3311,7 @@
       <c r="AE53" s="4"/>
       <c r="AF53" s="4"/>
     </row>
-    <row r="54" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B54" s="3" t="s">
         <v>55</v>
       </c>
@@ -3347,7 +3356,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="55" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B55" s="3" t="s">
         <v>56</v>
       </c>
@@ -3399,7 +3408,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="56" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B56" s="3" t="s">
         <v>56</v>
       </c>
@@ -3441,7 +3450,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="57" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B57" s="3" t="s">
         <v>56</v>
       </c>
@@ -3493,7 +3502,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="58" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B58" s="3" t="s">
         <v>56</v>
       </c>
@@ -3535,7 +3544,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="59" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B59" s="3" t="s">
         <v>56</v>
       </c>
@@ -3587,7 +3596,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="60" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B60" s="3" t="s">
         <v>56</v>
       </c>
@@ -3631,7 +3640,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="61" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B61" s="3" t="s">
         <v>56</v>
       </c>
@@ -3678,7 +3687,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="62" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B62" s="3" t="s">
         <v>56</v>
       </c>
@@ -3722,7 +3731,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="63" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B63" s="3" t="s">
         <v>57</v>
       </c>
@@ -3778,7 +3787,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="64" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B64" s="3" t="s">
         <v>57</v>
       </c>
@@ -3822,7 +3831,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="65" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B65" s="3" t="s">
         <v>57</v>
       </c>
@@ -3872,7 +3881,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="66" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B66" s="3" t="s">
         <v>57</v>
       </c>
@@ -3916,7 +3925,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="67" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B67" s="3" t="s">
         <v>57</v>
       </c>
@@ -3968,7 +3977,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="68" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B68" s="3" t="s">
         <v>57</v>
       </c>
@@ -4012,7 +4021,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="69" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B69" s="3" t="s">
         <v>58</v>
       </c>
@@ -4077,7 +4086,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="70" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B70" s="3" t="s">
         <v>58</v>
       </c>
@@ -4120,7 +4129,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="71" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B71" s="3" t="s">
         <v>58</v>
       </c>
@@ -4176,7 +4185,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="72" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B72" s="3" t="s">
         <v>58</v>
       </c>
@@ -4218,7 +4227,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="73" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B73" s="3" t="s">
         <v>58</v>
       </c>
@@ -4276,7 +4285,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="74" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B74" s="3" t="s">
         <v>58</v>
       </c>
@@ -4320,7 +4329,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="75" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B75" s="3" t="s">
         <v>59</v>
       </c>
@@ -4367,7 +4376,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="76" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B76" s="3" t="s">
         <v>59</v>
       </c>
@@ -4412,7 +4421,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="77" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B77" s="3" t="s">
         <v>59</v>
       </c>
@@ -4459,7 +4468,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="78" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B78" s="3" t="s">
         <v>59</v>
       </c>
@@ -4503,7 +4512,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="79" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B79" s="3" t="s">
         <v>60</v>
       </c>
@@ -4552,7 +4561,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="80" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B80" s="3" t="s">
         <v>60</v>
       </c>
@@ -4595,7 +4604,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="81" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B81" t="s">
         <v>61</v>
       </c>
@@ -4630,7 +4639,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="82" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B82" t="s">
         <v>61</v>
       </c>
@@ -4668,7 +4677,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="83" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B83" s="3" t="s">
         <v>62</v>
       </c>
@@ -4713,7 +4722,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="84" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B84" s="3" t="s">
         <v>62</v>
       </c>
@@ -4758,7 +4767,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="85" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B85" s="3" t="s">
         <v>62</v>
       </c>
@@ -4801,7 +4810,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="86" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B86" s="3" t="s">
         <v>62</v>
       </c>
@@ -4839,7 +4848,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="87" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B87" s="3" t="s">
         <v>62</v>
       </c>
@@ -4879,7 +4888,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="88" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B88" s="3" t="s">
         <v>62</v>
       </c>
@@ -4917,7 +4926,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="89" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B89" s="3" t="s">
         <v>62</v>
       </c>
@@ -4957,7 +4966,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="90" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B90" s="3" t="s">
         <v>62</v>
       </c>
@@ -4995,7 +5004,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="91" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B91" s="3" t="s">
         <v>62</v>
       </c>
@@ -5038,7 +5047,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="92" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B92" s="3" t="s">
         <v>62</v>
       </c>
@@ -5076,7 +5085,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="93" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B93" s="3" t="s">
         <v>62</v>
       </c>
@@ -5116,7 +5125,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="94" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B94" s="3" t="s">
         <v>62</v>
       </c>
@@ -5154,7 +5163,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="95" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B95" s="3" t="s">
         <v>62</v>
       </c>
@@ -5194,7 +5203,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="96" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B96" s="3" t="s">
         <v>62</v>
       </c>
@@ -5232,7 +5241,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="97" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B97" s="3" t="s">
         <v>62</v>
       </c>
@@ -5272,7 +5281,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="98" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B98" s="3" t="s">
         <v>62</v>
       </c>
@@ -5310,7 +5319,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="99" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B99" s="3" t="s">
         <v>62</v>
       </c>
@@ -5350,7 +5359,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="100" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B100" s="3" t="s">
         <v>62</v>
       </c>
@@ -5388,7 +5397,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="101" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B101" s="3" t="s">
         <v>62</v>
       </c>
@@ -5431,7 +5440,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="102" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B102" s="3" t="s">
         <v>62</v>
       </c>
@@ -5469,7 +5478,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="103" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B103" s="3" t="s">
         <v>62</v>
       </c>
@@ -5514,7 +5523,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="104" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B104" s="3" t="s">
         <v>62</v>
       </c>
@@ -5552,7 +5561,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="105" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B105" s="3" t="s">
         <v>62</v>
       </c>
@@ -5597,7 +5606,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="106" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:33" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B106" s="3" t="s">
         <v>62</v>
       </c>
@@ -5635,7 +5644,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="107" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B107" s="3" t="s">
         <v>62</v>
       </c>
@@ -5678,7 +5687,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="108" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B108" s="3" t="s">
         <v>62</v>
       </c>
@@ -5716,7 +5725,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="109" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B109" s="3" t="s">
         <v>62</v>
       </c>
@@ -5759,7 +5768,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="110" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B110" s="3" t="s">
         <v>62</v>
       </c>
@@ -5797,7 +5806,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="111" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B111" s="3" t="s">
         <v>62</v>
       </c>
@@ -5842,7 +5851,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="112" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B112" s="3" t="s">
         <v>62</v>
       </c>
@@ -5880,7 +5889,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="113" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B113" s="3" t="s">
         <v>62</v>
       </c>
@@ -5926,7 +5935,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="114" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B114" s="3" t="s">
         <v>62</v>
       </c>
@@ -5969,7 +5978,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="115" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B115" s="3" t="s">
         <v>63</v>
       </c>
@@ -6017,7 +6026,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="116" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B116" s="3" t="s">
         <v>63</v>
       </c>
@@ -6060,7 +6069,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="117" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B117" s="3" t="s">
         <v>63</v>
       </c>
@@ -6105,7 +6114,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="118" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B118" s="3" t="s">
         <v>63</v>
       </c>
@@ -6143,7 +6152,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="119" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B119" s="3" t="s">
         <v>63</v>
       </c>
@@ -6186,7 +6195,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="120" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B120" s="3" t="s">
         <v>63</v>
       </c>
@@ -6224,7 +6233,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="121" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B121" s="3" t="s">
         <v>63</v>
       </c>
@@ -6269,7 +6278,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="122" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="122" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B122" s="3" t="s">
         <v>63</v>
       </c>
@@ -6307,7 +6316,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="123" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B123" s="3" t="s">
         <v>63</v>
       </c>
@@ -6352,7 +6361,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="124" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B124" s="3" t="s">
         <v>63</v>
       </c>
@@ -6390,7 +6399,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="125" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="125" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B125" s="3" t="s">
         <v>63</v>
       </c>
@@ -6433,7 +6442,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="126" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B126" s="3" t="s">
         <v>63</v>
       </c>
@@ -6471,7 +6480,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="127" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="127" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B127" s="3" t="s">
         <v>63</v>
       </c>
@@ -6514,7 +6523,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="128" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B128" s="3" t="s">
         <v>63</v>
       </c>
@@ -6552,7 +6561,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="129" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B129" s="3" t="s">
         <v>63</v>
       </c>
@@ -6595,7 +6604,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="130" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B130" s="3" t="s">
         <v>63</v>
       </c>
@@ -6633,7 +6642,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="131" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="131" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B131" s="3" t="s">
         <v>63</v>
       </c>
@@ -6678,7 +6687,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="132" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="132" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B132" s="3" t="s">
         <v>63</v>
       </c>
@@ -6719,7 +6728,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="133" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="133" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B133" s="3" t="s">
         <v>64</v>
       </c>
@@ -6776,7 +6785,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="134" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="134" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B134" s="3" t="s">
         <v>64</v>
       </c>
@@ -6819,7 +6828,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="135" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="135" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B135" s="3" t="s">
         <v>64</v>
       </c>
@@ -6865,7 +6874,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="136" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="136" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B136" s="3" t="s">
         <v>64</v>
       </c>
@@ -6908,7 +6917,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="137" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="137" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B137" s="3" t="s">
         <v>64</v>
       </c>
@@ -6954,7 +6963,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="138" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="138" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B138" s="3" t="s">
         <v>64</v>
       </c>
@@ -6997,7 +7006,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="139" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="139" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B139" t="s">
         <v>65</v>
       </c>
@@ -7046,7 +7055,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="140" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="140" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B140" t="s">
         <v>65</v>
       </c>
@@ -7087,7 +7096,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="141" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="141" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B141" t="s">
         <v>65</v>
       </c>
@@ -7137,7 +7146,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="142" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="142" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B142" t="s">
         <v>65</v>
       </c>
@@ -7182,7 +7191,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="143" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="143" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B143" s="3" t="s">
         <v>66</v>
       </c>
@@ -7228,7 +7237,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="144" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="144" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B144" s="3" t="s">
         <v>66</v>
       </c>
@@ -7266,7 +7275,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="145" spans="2:38" x14ac:dyDescent="0.3">
+    <row r="145" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
       <c r="B145" t="s">
         <v>67</v>
       </c>
@@ -7304,7 +7313,7 @@
       <c r="AE145" s="4"/>
       <c r="AF145" s="4"/>
     </row>
-    <row r="146" spans="2:38" x14ac:dyDescent="0.3">
+    <row r="146" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
       <c r="B146" t="s">
         <v>67</v>
       </c>
@@ -7339,7 +7348,7 @@
       <c r="AE146" s="4"/>
       <c r="AF146" s="4"/>
     </row>
-    <row r="147" spans="2:38" x14ac:dyDescent="0.3">
+    <row r="147" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
       <c r="B147" t="s">
         <v>68</v>
       </c>
@@ -7374,7 +7383,7 @@
       <c r="AE147" s="4"/>
       <c r="AF147" s="4"/>
     </row>
-    <row r="148" spans="2:38" x14ac:dyDescent="0.3">
+    <row r="148" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
       <c r="B148" t="s">
         <v>68</v>
       </c>
@@ -7409,7 +7418,7 @@
       <c r="AE148" s="4"/>
       <c r="AF148" s="4"/>
     </row>
-    <row r="149" spans="2:38" x14ac:dyDescent="0.3">
+    <row r="149" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
       <c r="B149" t="s">
         <v>69</v>
       </c>
@@ -7450,7 +7459,7 @@
       <c r="AE149" s="4"/>
       <c r="AF149" s="4"/>
     </row>
-    <row r="150" spans="2:38" x14ac:dyDescent="0.3">
+    <row r="150" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
       <c r="B150" t="s">
         <v>69</v>
       </c>
@@ -7464,7 +7473,7 @@
         <v>1799.2</v>
       </c>
       <c r="F150" s="3">
-        <v>1403.2</v>
+        <v>1432.2</v>
       </c>
       <c r="L150" s="4"/>
       <c r="M150" s="4"/>
@@ -7483,7 +7492,7 @@
         <v>888</v>
       </c>
       <c r="Z150" s="4">
-        <v>515.20000000000005</v>
+        <v>544.20000000000005</v>
       </c>
       <c r="AA150" s="4"/>
       <c r="AB150" s="4"/>
@@ -7495,7 +7504,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="151" spans="2:38" x14ac:dyDescent="0.3">
+    <row r="151" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
       <c r="B151" t="s">
         <v>70</v>
       </c>
@@ -7527,7 +7536,7 @@
       <c r="AE151" s="4"/>
       <c r="AF151" s="4"/>
     </row>
-    <row r="152" spans="2:38" x14ac:dyDescent="0.3">
+    <row r="152" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
       <c r="B152" t="s">
         <v>70</v>
       </c>
@@ -7562,7 +7571,7 @@
       <c r="AE152" s="4"/>
       <c r="AF152" s="4"/>
     </row>
-    <row r="153" spans="2:38" x14ac:dyDescent="0.3">
+    <row r="153" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
       <c r="B153" t="s">
         <v>71</v>
       </c>
@@ -7597,7 +7606,7 @@
       <c r="AE153" s="4"/>
       <c r="AF153" s="4"/>
     </row>
-    <row r="154" spans="2:38" x14ac:dyDescent="0.3">
+    <row r="154" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
       <c r="B154" t="s">
         <v>71</v>
       </c>
@@ -7632,7 +7641,7 @@
       <c r="AE154" s="4"/>
       <c r="AF154" s="4"/>
     </row>
-    <row r="155" spans="2:38" x14ac:dyDescent="0.3">
+    <row r="155" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
       <c r="B155" t="s">
         <v>72</v>
       </c>
@@ -7670,7 +7679,7 @@
         <v>1746.61</v>
       </c>
     </row>
-    <row r="156" spans="2:38" x14ac:dyDescent="0.3">
+    <row r="156" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
       <c r="B156" t="s">
         <v>72</v>
       </c>
@@ -7708,7 +7717,7 @@
         <v>1471.49</v>
       </c>
     </row>
-    <row r="157" spans="2:38" x14ac:dyDescent="0.3">
+    <row r="157" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
       <c r="B157" t="s">
         <v>73</v>
       </c>
@@ -7747,7 +7756,7 @@
         <v>275.11999999999989</v>
       </c>
     </row>
-    <row r="158" spans="2:38" x14ac:dyDescent="0.3">
+    <row r="158" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
       <c r="B158" t="s">
         <v>73</v>
       </c>
@@ -7782,7 +7791,7 @@
       <c r="AE158" s="4"/>
       <c r="AF158" s="4"/>
     </row>
-    <row r="159" spans="2:38" x14ac:dyDescent="0.3">
+    <row r="159" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
       <c r="B159" s="3" t="s">
         <v>75</v>
       </c>
@@ -7843,7 +7852,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="160" spans="2:38" x14ac:dyDescent="0.3">
+    <row r="160" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
       <c r="B160" s="3" t="s">
         <v>75</v>
       </c>
@@ -7896,7 +7905,7 @@
         <v>91.706666666666635</v>
       </c>
     </row>
-    <row r="161" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="161" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B161" s="3" t="s">
         <v>75</v>
       </c>
@@ -7955,7 +7964,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="162" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="162" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B162" s="3" t="s">
         <v>75</v>
       </c>
@@ -8001,7 +8010,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="163" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="163" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B163" s="3" t="s">
         <v>75</v>
       </c>
@@ -8050,7 +8059,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="164" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="164" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B164" s="3" t="s">
         <v>75</v>
       </c>
@@ -8093,7 +8102,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="165" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="165" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B165" t="s">
         <v>76</v>
       </c>
@@ -8131,7 +8140,7 @@
       <c r="AE165" s="4"/>
       <c r="AF165" s="4"/>
     </row>
-    <row r="166" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="166" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B166" t="s">
         <v>76</v>
       </c>
@@ -8166,7 +8175,7 @@
       <c r="AE166" s="4"/>
       <c r="AF166" s="4"/>
     </row>
-    <row r="167" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="167" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B167" t="s">
         <v>77</v>
       </c>
@@ -8198,7 +8207,7 @@
       <c r="AE167" s="4"/>
       <c r="AF167" s="4"/>
     </row>
-    <row r="168" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="168" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B168" t="s">
         <v>77</v>
       </c>
@@ -8233,7 +8242,7 @@
       <c r="AE168" s="4"/>
       <c r="AF168" s="4"/>
     </row>
-    <row r="169" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="169" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B169" s="3" t="s">
         <v>78</v>
       </c>
@@ -8279,7 +8288,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="170" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="170" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B170" s="3" t="s">
         <v>78</v>
       </c>
@@ -8317,7 +8326,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="171" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="171" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B171" s="3" t="s">
         <v>78</v>
       </c>
@@ -8366,7 +8375,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="172" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="172" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B172" s="3" t="s">
         <v>78</v>
       </c>
@@ -8409,7 +8418,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="173" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="173" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B173" t="s">
         <v>79</v>
       </c>
@@ -8447,7 +8456,7 @@
       <c r="AE173" s="4"/>
       <c r="AF173" s="4"/>
     </row>
-    <row r="174" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="174" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B174" t="s">
         <v>79</v>
       </c>
@@ -8482,7 +8491,7 @@
       <c r="AE174" s="4"/>
       <c r="AF174" s="4"/>
     </row>
-    <row r="175" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="175" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B175" t="s">
         <v>80</v>
       </c>
@@ -8514,7 +8523,7 @@
       <c r="AE175" s="4"/>
       <c r="AF175" s="4"/>
     </row>
-    <row r="176" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="176" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B176" t="s">
         <v>80</v>
       </c>
@@ -8549,7 +8558,7 @@
       <c r="AE176" s="4"/>
       <c r="AF176" s="4"/>
     </row>
-    <row r="177" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="177" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B177" t="s">
         <v>81</v>
       </c>
@@ -8587,7 +8596,7 @@
       <c r="AE177" s="4"/>
       <c r="AF177" s="4"/>
     </row>
-    <row r="178" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="178" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B178" t="s">
         <v>81</v>
       </c>
@@ -8622,7 +8631,7 @@
       <c r="AE178" s="4"/>
       <c r="AF178" s="4"/>
     </row>
-    <row r="179" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="179" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B179" t="s">
         <v>82</v>
       </c>
@@ -8654,7 +8663,7 @@
       <c r="AE179" s="4"/>
       <c r="AF179" s="4"/>
     </row>
-    <row r="180" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="180" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B180" t="s">
         <v>82</v>
       </c>
@@ -8689,7 +8698,7 @@
       <c r="AE180" s="4"/>
       <c r="AF180" s="4"/>
     </row>
-    <row r="181" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="181" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B181" s="3" t="s">
         <v>83</v>
       </c>
@@ -8738,7 +8747,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="182" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="182" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B182" s="3" t="s">
         <v>83</v>
       </c>
@@ -8782,7 +8791,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="183" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="183" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B183" t="s">
         <v>84</v>
       </c>
@@ -8817,7 +8826,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="184" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="184" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B184" t="s">
         <v>84</v>
       </c>
@@ -8857,7 +8866,7 @@
       <c r="AE184" s="4"/>
       <c r="AF184" s="4"/>
     </row>
-    <row r="185" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="185" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B185" t="s">
         <v>85</v>
       </c>
@@ -8895,7 +8904,7 @@
       <c r="AE185" s="4"/>
       <c r="AF185" s="4"/>
     </row>
-    <row r="186" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="186" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B186" t="s">
         <v>85</v>
       </c>
@@ -8930,7 +8939,7 @@
       <c r="AE186" s="4"/>
       <c r="AF186" s="4"/>
     </row>
-    <row r="187" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="187" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B187" t="s">
         <v>86</v>
       </c>
@@ -8965,7 +8974,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="188" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="188" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B188" t="s">
         <v>86</v>
       </c>
@@ -9008,7 +9017,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="189" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="189" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B189" t="s">
         <v>87</v>
       </c>
@@ -9040,7 +9049,7 @@
       <c r="AE189" s="4"/>
       <c r="AF189" s="4"/>
     </row>
-    <row r="190" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="190" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B190" t="s">
         <v>87</v>
       </c>
@@ -9075,7 +9084,7 @@
       <c r="AE190" s="4"/>
       <c r="AF190" s="4"/>
     </row>
-    <row r="191" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="191" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B191" t="s">
         <v>88</v>
       </c>
@@ -9107,7 +9116,7 @@
       <c r="AE191" s="4"/>
       <c r="AF191" s="4"/>
     </row>
-    <row r="192" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="192" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B192" t="s">
         <v>88</v>
       </c>
@@ -9142,7 +9151,7 @@
       <c r="AE192" s="4"/>
       <c r="AF192" s="4"/>
     </row>
-    <row r="193" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="193" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B193" t="s">
         <v>89</v>
       </c>
@@ -9174,7 +9183,7 @@
       <c r="AE193" s="4"/>
       <c r="AF193" s="4"/>
     </row>
-    <row r="194" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="194" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B194" t="s">
         <v>89</v>
       </c>
@@ -9209,7 +9218,7 @@
       <c r="AE194" s="4"/>
       <c r="AF194" s="4"/>
     </row>
-    <row r="195" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="195" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B195" t="s">
         <v>90</v>
       </c>
@@ -9253,7 +9262,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="196" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="196" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B196" t="s">
         <v>90</v>
       </c>
@@ -9291,7 +9300,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="197" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="197" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B197" t="s">
         <v>91</v>
       </c>
@@ -9326,7 +9335,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="198" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="198" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B198" t="s">
         <v>91</v>
       </c>
@@ -9364,7 +9373,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="199" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="199" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B199" t="s">
         <v>92</v>
       </c>
@@ -9399,7 +9408,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="200" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="200" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B200" t="s">
         <v>92</v>
       </c>
@@ -9478,6 +9487,9 @@
       <c r="AD201" s="4"/>
       <c r="AE201" s="4"/>
       <c r="AF201" s="4"/>
+      <c r="AG201" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="202" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B202" t="s">
@@ -9513,8 +9525,11 @@
       <c r="AD202" s="4"/>
       <c r="AE202" s="4"/>
       <c r="AF202" s="4"/>
-    </row>
-    <row r="203" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG202" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="203" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B203" t="s">
         <v>94</v>
       </c>
@@ -9546,7 +9561,7 @@
       <c r="AE203" s="4"/>
       <c r="AF203" s="4"/>
     </row>
-    <row r="204" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="204" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B204" t="s">
         <v>94</v>
       </c>
@@ -9581,7 +9596,7 @@
       <c r="AE204" s="4"/>
       <c r="AF204" s="4"/>
     </row>
-    <row r="205" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="205" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B205" t="s">
         <v>95</v>
       </c>
@@ -9621,7 +9636,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="206" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="206" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B206" t="s">
         <v>95</v>
       </c>
@@ -9656,7 +9671,7 @@
       <c r="AE206" s="4"/>
       <c r="AF206" s="4"/>
     </row>
-    <row r="207" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="207" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B207" t="s">
         <v>96</v>
       </c>
@@ -9691,7 +9706,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="208" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="208" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B208" t="s">
         <v>96</v>
       </c>
@@ -9736,7 +9751,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="209" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="209" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B209" s="3" t="s">
         <v>62</v>
       </c>
@@ -9779,7 +9794,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="210" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="210" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B210" s="3" t="s">
         <v>62</v>
       </c>
@@ -9817,7 +9832,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="211" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="211" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B211" t="s">
         <v>98</v>
       </c>
@@ -9863,7 +9878,7 @@
       <c r="AE211" s="4"/>
       <c r="AF211" s="4"/>
     </row>
-    <row r="212" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="212" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B212" t="s">
         <v>98</v>
       </c>
@@ -9907,7 +9922,7 @@
       <c r="AE212" s="4"/>
       <c r="AF212" s="4"/>
     </row>
-    <row r="213" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="213" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B213" t="s">
         <v>100</v>
       </c>
@@ -9942,7 +9957,7 @@
       <c r="AE213" s="4"/>
       <c r="AF213" s="4"/>
     </row>
-    <row r="214" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="214" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B214" t="s">
         <v>100</v>
       </c>
@@ -9977,7 +9992,7 @@
       <c r="AE214" s="4"/>
       <c r="AF214" s="4"/>
     </row>
-    <row r="215" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="215" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B215" t="s">
         <v>102</v>
       </c>
@@ -10012,7 +10027,7 @@
       <c r="AE215" s="4"/>
       <c r="AF215" s="4"/>
     </row>
-    <row r="216" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="216" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B216" t="s">
         <v>102</v>
       </c>
@@ -10047,7 +10062,7 @@
       <c r="AE216" s="4"/>
       <c r="AF216" s="4"/>
     </row>
-    <row r="217" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="217" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B217" t="s">
         <v>104</v>
       </c>
@@ -10079,7 +10094,7 @@
       <c r="AE217" s="4"/>
       <c r="AF217" s="4"/>
     </row>
-    <row r="218" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="218" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B218" t="s">
         <v>104</v>
       </c>

</xml_diff>

<commit_message>
Atualiza extensao e EAP novamente
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FFBE20F-9C81-4ABA-8E0B-45582CC3C91A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DED96A70-3D12-4F17-AEF2-A3ACCDE3CC73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BASE_DASH_EXTENSAO" sheetId="1" r:id="rId1"/>
@@ -9436,7 +9436,7 @@
         <v>180</v>
       </c>
       <c r="F200" s="3">
-        <v>160.86000000000001</v>
+        <v>167.96</v>
       </c>
       <c r="L200" s="4"/>
       <c r="M200" s="4"/>
@@ -9455,9 +9455,11 @@
         <v>43.66</v>
       </c>
       <c r="Z200" s="9">
-        <v>198.8</v>
-      </c>
-      <c r="AA200" s="4"/>
+        <v>89.8</v>
+      </c>
+      <c r="AA200" s="4">
+        <v>34.5</v>
+      </c>
       <c r="AB200" s="4"/>
       <c r="AC200" s="4"/>
       <c r="AD200" s="4"/>

</xml_diff>

<commit_message>
Atualiza EAP extensao e PDS de 15 julho
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CD004AC-E1EE-4D7E-B6E0-236C936CEFF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA143249-3D47-4B4D-89D2-DB81D518D575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -799,13 +799,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tb_base_dash_extensao" displayName="tb_base_dash_extensao" ref="B1:AF218">
-  <autoFilter ref="B1:AF218" xr:uid="{00000000-0009-0000-0100-000001000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="RCE COMUNIDADE JD. UNIÃO"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="B1:AF218" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:AF218">
     <sortCondition ref="B1:B218"/>
   </sortState>
@@ -1259,7 +1253,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B2" s="3" t="s">
         <v>64</v>
       </c>
@@ -1316,7 +1310,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B3" s="3" t="s">
         <v>64</v>
       </c>
@@ -1359,7 +1353,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>64</v>
       </c>
@@ -1405,7 +1399,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B5" s="3" t="s">
         <v>64</v>
       </c>
@@ -1448,7 +1442,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
         <v>64</v>
       </c>
@@ -1494,7 +1488,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B7" s="3" t="s">
         <v>64</v>
       </c>
@@ -1537,7 +1531,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B8" s="3" t="s">
         <v>63</v>
       </c>
@@ -1585,7 +1579,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B9" s="3" t="s">
         <v>63</v>
       </c>
@@ -1628,7 +1622,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B10" s="3" t="s">
         <v>63</v>
       </c>
@@ -1673,7 +1667,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B11" s="3" t="s">
         <v>63</v>
       </c>
@@ -1711,7 +1705,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B12" s="3" t="s">
         <v>63</v>
       </c>
@@ -1754,7 +1748,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B13" s="3" t="s">
         <v>63</v>
       </c>
@@ -1792,7 +1786,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
         <v>63</v>
       </c>
@@ -1837,7 +1831,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B15" s="3" t="s">
         <v>63</v>
       </c>
@@ -1875,7 +1869,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
         <v>63</v>
       </c>
@@ -1920,7 +1914,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B17" s="3" t="s">
         <v>63</v>
       </c>
@@ -1958,7 +1952,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="18" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B18" s="3" t="s">
         <v>63</v>
       </c>
@@ -2001,7 +1995,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B19" s="3" t="s">
         <v>63</v>
       </c>
@@ -2039,7 +2033,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B20" s="3" t="s">
         <v>63</v>
       </c>
@@ -2082,7 +2076,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="21" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B21" s="3" t="s">
         <v>63</v>
       </c>
@@ -2120,7 +2114,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B22" s="3" t="s">
         <v>63</v>
       </c>
@@ -2163,7 +2157,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B23" s="3" t="s">
         <v>63</v>
       </c>
@@ -2201,7 +2195,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="24" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B24" s="3" t="s">
         <v>63</v>
       </c>
@@ -2246,7 +2240,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="25" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B25" s="3" t="s">
         <v>63</v>
       </c>
@@ -2287,7 +2281,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="26" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B26" s="3" t="s">
         <v>62</v>
       </c>
@@ -2329,7 +2323,7 @@
       <c r="AE26" s="4"/>
       <c r="AF26" s="4"/>
     </row>
-    <row r="27" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B27" s="3" t="s">
         <v>62</v>
       </c>
@@ -2371,7 +2365,7 @@
       <c r="AE27" s="4"/>
       <c r="AF27" s="4"/>
     </row>
-    <row r="28" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B28" s="3" t="s">
         <v>62</v>
       </c>
@@ -2411,7 +2405,7 @@
       <c r="AE28" s="4"/>
       <c r="AF28" s="4"/>
     </row>
-    <row r="29" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
         <v>62</v>
       </c>
@@ -2446,7 +2440,7 @@
       <c r="AE29" s="4"/>
       <c r="AF29" s="4"/>
     </row>
-    <row r="30" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B30" s="3" t="s">
         <v>62</v>
       </c>
@@ -2483,7 +2477,7 @@
       <c r="AE30" s="4"/>
       <c r="AF30" s="4"/>
     </row>
-    <row r="31" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B31" s="3" t="s">
         <v>62</v>
       </c>
@@ -2518,7 +2512,7 @@
       <c r="AE31" s="4"/>
       <c r="AF31" s="4"/>
     </row>
-    <row r="32" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B32" s="3" t="s">
         <v>62</v>
       </c>
@@ -2558,7 +2552,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="33" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B33" s="3" t="s">
         <v>62</v>
       </c>
@@ -2596,7 +2590,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="34" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B34" s="3" t="s">
         <v>62</v>
       </c>
@@ -2636,7 +2630,7 @@
       <c r="AE34" s="4"/>
       <c r="AF34" s="4"/>
     </row>
-    <row r="35" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B35" s="3" t="s">
         <v>62</v>
       </c>
@@ -2671,7 +2665,7 @@
       <c r="AE35" s="4"/>
       <c r="AF35" s="4"/>
     </row>
-    <row r="36" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B36" s="3" t="s">
         <v>62</v>
       </c>
@@ -2708,7 +2702,7 @@
       <c r="AE36" s="4"/>
       <c r="AF36" s="4"/>
     </row>
-    <row r="37" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B37" s="3" t="s">
         <v>62</v>
       </c>
@@ -2743,7 +2737,7 @@
       <c r="AE37" s="4"/>
       <c r="AF37" s="4"/>
     </row>
-    <row r="38" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B38" s="3" t="s">
         <v>62</v>
       </c>
@@ -2783,7 +2777,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="39" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B39" s="3" t="s">
         <v>62</v>
       </c>
@@ -2818,7 +2812,7 @@
       <c r="AE39" s="4"/>
       <c r="AF39" s="4"/>
     </row>
-    <row r="40" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B40" s="3" t="s">
         <v>62</v>
       </c>
@@ -2855,7 +2849,7 @@
       <c r="AE40" s="4"/>
       <c r="AF40" s="4"/>
     </row>
-    <row r="41" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B41" s="3" t="s">
         <v>62</v>
       </c>
@@ -2890,7 +2884,7 @@
       <c r="AE41" s="4"/>
       <c r="AF41" s="4"/>
     </row>
-    <row r="42" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B42" s="3" t="s">
         <v>62</v>
       </c>
@@ -2927,7 +2921,7 @@
       <c r="AE42" s="4"/>
       <c r="AF42" s="4"/>
     </row>
-    <row r="43" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B43" s="3" t="s">
         <v>62</v>
       </c>
@@ -2962,7 +2956,7 @@
       <c r="AE43" s="4"/>
       <c r="AF43" s="4"/>
     </row>
-    <row r="44" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B44" s="3" t="s">
         <v>62</v>
       </c>
@@ -3002,7 +2996,7 @@
       <c r="AE44" s="4"/>
       <c r="AF44" s="4"/>
     </row>
-    <row r="45" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B45" s="3" t="s">
         <v>62</v>
       </c>
@@ -3037,7 +3031,7 @@
       <c r="AE45" s="4"/>
       <c r="AF45" s="4"/>
     </row>
-    <row r="46" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B46" s="3" t="s">
         <v>62</v>
       </c>
@@ -3079,7 +3073,7 @@
       <c r="AE46" s="4"/>
       <c r="AF46" s="4"/>
     </row>
-    <row r="47" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B47" s="3" t="s">
         <v>62</v>
       </c>
@@ -3114,7 +3108,7 @@
       <c r="AE47" s="4"/>
       <c r="AF47" s="4"/>
     </row>
-    <row r="48" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B48" s="3" t="s">
         <v>62</v>
       </c>
@@ -3156,7 +3150,7 @@
       <c r="AE48" s="4"/>
       <c r="AF48" s="4"/>
     </row>
-    <row r="49" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B49" s="3" t="s">
         <v>62</v>
       </c>
@@ -3191,7 +3185,7 @@
       <c r="AE49" s="4"/>
       <c r="AF49" s="4"/>
     </row>
-    <row r="50" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B50" s="3" t="s">
         <v>62</v>
       </c>
@@ -3231,7 +3225,7 @@
       <c r="AE50" s="4"/>
       <c r="AF50" s="4"/>
     </row>
-    <row r="51" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B51" s="3" t="s">
         <v>62</v>
       </c>
@@ -3266,7 +3260,7 @@
       <c r="AE51" s="4"/>
       <c r="AF51" s="4"/>
     </row>
-    <row r="52" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B52" s="3" t="s">
         <v>62</v>
       </c>
@@ -3306,7 +3300,7 @@
       <c r="AE52" s="4"/>
       <c r="AF52" s="4"/>
     </row>
-    <row r="53" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B53" s="3" t="s">
         <v>62</v>
       </c>
@@ -3341,7 +3335,7 @@
       <c r="AE53" s="4"/>
       <c r="AF53" s="4"/>
     </row>
-    <row r="54" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B54" s="3" t="s">
         <v>62</v>
       </c>
@@ -3386,7 +3380,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="55" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B55" s="3" t="s">
         <v>62</v>
       </c>
@@ -3424,7 +3418,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="56" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B56" s="3" t="s">
         <v>62</v>
       </c>
@@ -3470,7 +3464,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="57" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B57" s="3" t="s">
         <v>62</v>
       </c>
@@ -3513,7 +3507,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="58" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B58" s="3" t="s">
         <v>62</v>
       </c>
@@ -3556,7 +3550,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="59" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B59" s="3" t="s">
         <v>62</v>
       </c>
@@ -3594,7 +3588,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="60" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B60" s="3" t="s">
         <v>58</v>
       </c>
@@ -3659,7 +3653,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="61" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B61" s="3" t="s">
         <v>58</v>
       </c>
@@ -3702,7 +3696,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="62" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B62" s="3" t="s">
         <v>58</v>
       </c>
@@ -3758,7 +3752,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="63" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B63" s="3" t="s">
         <v>58</v>
       </c>
@@ -3800,7 +3794,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="64" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B64" s="3" t="s">
         <v>58</v>
       </c>
@@ -3858,7 +3852,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="65" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B65" s="3" t="s">
         <v>58</v>
       </c>
@@ -3902,7 +3896,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="66" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B66" s="3" t="s">
         <v>59</v>
       </c>
@@ -3949,7 +3943,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="67" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B67" s="3" t="s">
         <v>59</v>
       </c>
@@ -3994,7 +3988,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="68" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B68" s="3" t="s">
         <v>59</v>
       </c>
@@ -4041,7 +4035,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="69" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B69" s="3" t="s">
         <v>59</v>
       </c>
@@ -4085,7 +4079,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="70" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B70" s="3" t="s">
         <v>33</v>
       </c>
@@ -4131,7 +4125,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="71" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B71" s="3" t="s">
         <v>33</v>
       </c>
@@ -4174,7 +4168,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="72" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B72" s="3" t="s">
         <v>33</v>
       </c>
@@ -4219,7 +4213,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="73" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B73" s="3" t="s">
         <v>33</v>
       </c>
@@ -4262,7 +4256,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="74" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B74" s="3" t="s">
         <v>33</v>
       </c>
@@ -4305,7 +4299,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="75" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B75" s="3" t="s">
         <v>33</v>
       </c>
@@ -4348,7 +4342,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="76" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B76" s="3" t="s">
         <v>33</v>
       </c>
@@ -4396,7 +4390,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="77" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B77" s="3" t="s">
         <v>33</v>
       </c>
@@ -4440,7 +4434,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="78" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B78" s="3" t="s">
         <v>38</v>
       </c>
@@ -4495,7 +4489,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="79" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B79" s="3" t="s">
         <v>38</v>
       </c>
@@ -4538,7 +4532,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="80" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B80" s="3" t="s">
         <v>38</v>
       </c>
@@ -4587,7 +4581,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="81" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B81" s="3" t="s">
         <v>38</v>
       </c>
@@ -4630,7 +4624,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="82" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B82" s="3" t="s">
         <v>60</v>
       </c>
@@ -4679,7 +4673,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="83" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B83" s="3" t="s">
         <v>60</v>
       </c>
@@ -4722,7 +4716,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="84" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B84" s="3" t="s">
         <v>57</v>
       </c>
@@ -4778,7 +4772,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="85" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B85" s="3" t="s">
         <v>57</v>
       </c>
@@ -4822,7 +4816,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="86" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B86" s="3" t="s">
         <v>57</v>
       </c>
@@ -4872,7 +4866,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="87" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B87" s="3" t="s">
         <v>57</v>
       </c>
@@ -4916,7 +4910,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="88" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B88" s="3" t="s">
         <v>57</v>
       </c>
@@ -4968,7 +4962,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="89" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B89" s="3" t="s">
         <v>57</v>
       </c>
@@ -5012,7 +5006,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="90" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B90" t="s">
         <v>52</v>
       </c>
@@ -5050,7 +5044,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="91" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B91" t="s">
         <v>52</v>
       </c>
@@ -5088,7 +5082,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="92" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B92" s="3" t="s">
         <v>56</v>
       </c>
@@ -5140,7 +5134,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="93" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B93" s="3" t="s">
         <v>56</v>
       </c>
@@ -5182,7 +5176,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="94" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B94" s="3" t="s">
         <v>56</v>
       </c>
@@ -5234,7 +5228,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="95" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B95" s="3" t="s">
         <v>56</v>
       </c>
@@ -5276,7 +5270,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="96" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B96" s="3" t="s">
         <v>56</v>
       </c>
@@ -5328,7 +5322,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="97" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B97" s="3" t="s">
         <v>56</v>
       </c>
@@ -5372,7 +5366,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="98" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B98" s="3" t="s">
         <v>56</v>
       </c>
@@ -5419,7 +5413,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="99" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B99" s="3" t="s">
         <v>56</v>
       </c>
@@ -5463,7 +5457,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="100" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B100" s="3" t="s">
         <v>55</v>
       </c>
@@ -5510,7 +5504,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="101" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B101" s="3" t="s">
         <v>37</v>
       </c>
@@ -5567,7 +5561,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="102" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B102" s="3" t="s">
         <v>37</v>
       </c>
@@ -5605,7 +5599,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="103" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B103" s="3" t="s">
         <v>37</v>
       </c>
@@ -5656,7 +5650,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="104" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B104" s="3" t="s">
         <v>37</v>
       </c>
@@ -5697,7 +5691,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="105" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B105" s="3" t="s">
         <v>37</v>
       </c>
@@ -5748,7 +5742,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="106" spans="2:33" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B106" s="3" t="s">
         <v>37</v>
       </c>
@@ -5791,7 +5785,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="107" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B107" s="3" t="s">
         <v>37</v>
       </c>
@@ -5844,7 +5838,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="108" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B108" s="3" t="s">
         <v>37</v>
       </c>
@@ -5882,7 +5876,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="109" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B109" s="3" t="s">
         <v>37</v>
       </c>
@@ -5931,7 +5925,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="110" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B110" s="3" t="s">
         <v>37</v>
       </c>
@@ -5980,7 +5974,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="111" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B111" t="s">
         <v>89</v>
       </c>
@@ -6024,7 +6018,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="112" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B112" t="s">
         <v>89</v>
       </c>
@@ -6062,7 +6056,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="113" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B113" s="3" t="s">
         <v>77</v>
       </c>
@@ -6108,7 +6102,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="114" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B114" s="3" t="s">
         <v>77</v>
       </c>
@@ -6146,7 +6140,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="115" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B115" s="3" t="s">
         <v>77</v>
       </c>
@@ -6195,7 +6189,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="116" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B116" s="3" t="s">
         <v>77</v>
       </c>
@@ -6238,7 +6232,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="117" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B117" s="3" t="s">
         <v>74</v>
       </c>
@@ -6299,7 +6293,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="118" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B118" s="3" t="s">
         <v>74</v>
       </c>
@@ -6348,7 +6342,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="119" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B119" s="3" t="s">
         <v>74</v>
       </c>
@@ -6407,7 +6401,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="120" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B120" s="3" t="s">
         <v>74</v>
       </c>
@@ -6453,7 +6447,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="121" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B121" s="3" t="s">
         <v>74</v>
       </c>
@@ -6502,7 +6496,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="122" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B122" s="3" t="s">
         <v>74</v>
       </c>
@@ -6545,7 +6539,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="123" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B123" t="s">
         <v>50</v>
       </c>
@@ -6583,7 +6577,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="124" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B124" t="s">
         <v>50</v>
       </c>
@@ -6618,7 +6612,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="125" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B125" t="s">
         <v>53</v>
       </c>
@@ -6656,7 +6650,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="126" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B126" t="s">
         <v>53</v>
       </c>
@@ -6694,7 +6688,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="127" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B127" t="s">
         <v>48</v>
       </c>
@@ -6732,7 +6726,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="128" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B128" t="s">
         <v>48</v>
       </c>
@@ -6767,7 +6761,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="129" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B129" t="s">
         <v>70</v>
       </c>
@@ -6802,7 +6796,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="130" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B130" t="s">
         <v>70</v>
       </c>
@@ -6840,7 +6834,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="131" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B131" s="3" t="s">
         <v>82</v>
       </c>
@@ -6889,7 +6883,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="132" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B132" s="3" t="s">
         <v>82</v>
       </c>
@@ -6933,7 +6927,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="133" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B133" t="s">
         <v>71</v>
       </c>
@@ -6971,7 +6965,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="134" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B134" t="s">
         <v>71</v>
       </c>
@@ -7014,7 +7008,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="135" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B135" t="s">
         <v>80</v>
       </c>
@@ -7055,7 +7049,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="136" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B136" t="s">
         <v>80</v>
       </c>
@@ -7093,7 +7087,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="137" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B137" t="s">
         <v>51</v>
       </c>
@@ -7131,7 +7125,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="138" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B138" t="s">
         <v>51</v>
       </c>
@@ -7169,7 +7163,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="139" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B139" t="s">
         <v>49</v>
       </c>
@@ -7207,7 +7201,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="140" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B140" t="s">
         <v>49</v>
       </c>
@@ -7242,7 +7236,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="141" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B141" t="s">
         <v>81</v>
       </c>
@@ -7277,7 +7271,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="142" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B142" t="s">
         <v>81</v>
       </c>
@@ -7315,7 +7309,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="143" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B143" t="s">
         <v>47</v>
       </c>
@@ -7350,7 +7344,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="144" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B144" t="s">
         <v>47</v>
       </c>
@@ -7395,7 +7389,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="145" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B145" t="s">
         <v>65</v>
       </c>
@@ -7441,7 +7435,7 @@
       <c r="AE145" s="4"/>
       <c r="AF145" s="4"/>
     </row>
-    <row r="146" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B146" t="s">
         <v>65</v>
       </c>
@@ -7479,7 +7473,7 @@
       <c r="AE146" s="4"/>
       <c r="AF146" s="4"/>
     </row>
-    <row r="147" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B147" t="s">
         <v>65</v>
       </c>
@@ -7526,7 +7520,7 @@
       <c r="AE147" s="4"/>
       <c r="AF147" s="4"/>
     </row>
-    <row r="148" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B148" t="s">
         <v>65</v>
       </c>
@@ -7568,7 +7562,7 @@
       <c r="AE148" s="4"/>
       <c r="AF148" s="4"/>
     </row>
-    <row r="149" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B149" t="s">
         <v>79</v>
       </c>
@@ -7600,7 +7594,7 @@
       <c r="AE149" s="4"/>
       <c r="AF149" s="4"/>
     </row>
-    <row r="150" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B150" t="s">
         <v>79</v>
       </c>
@@ -7638,7 +7632,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="151" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B151" s="3" t="s">
         <v>66</v>
       </c>
@@ -7681,7 +7675,7 @@
       <c r="AE151" s="4"/>
       <c r="AF151" s="4"/>
     </row>
-    <row r="152" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B152" s="3" t="s">
         <v>66</v>
       </c>
@@ -7716,7 +7710,7 @@
       <c r="AE152" s="4"/>
       <c r="AF152" s="4"/>
     </row>
-    <row r="153" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B153" t="s">
         <v>67</v>
       </c>
@@ -7754,7 +7748,7 @@
       <c r="AE153" s="4"/>
       <c r="AF153" s="4"/>
     </row>
-    <row r="154" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B154" t="s">
         <v>67</v>
       </c>
@@ -7789,7 +7783,7 @@
       <c r="AE154" s="4"/>
       <c r="AF154" s="4"/>
     </row>
-    <row r="155" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B155" t="s">
         <v>86</v>
       </c>
@@ -7824,7 +7818,7 @@
         <v>1746.61</v>
       </c>
     </row>
-    <row r="156" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B156" t="s">
         <v>86</v>
       </c>
@@ -7862,7 +7856,7 @@
         <v>1471.49</v>
       </c>
     </row>
-    <row r="157" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B157" t="s">
         <v>87</v>
       </c>
@@ -7898,7 +7892,7 @@
         <v>275.11999999999989</v>
       </c>
     </row>
-    <row r="158" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B158" t="s">
         <v>87</v>
       </c>
@@ -7933,7 +7927,7 @@
       <c r="AE158" s="4"/>
       <c r="AF158" s="4"/>
     </row>
-    <row r="159" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B159" t="s">
         <v>88</v>
       </c>
@@ -7968,7 +7962,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="160" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B160" t="s">
         <v>88</v>
       </c>
@@ -8010,7 +8004,7 @@
         <v>91.706666666666635</v>
       </c>
     </row>
-    <row r="161" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B161" t="s">
         <v>76</v>
       </c>
@@ -8045,7 +8039,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="162" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B162" t="s">
         <v>76</v>
       </c>
@@ -8083,7 +8077,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="163" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B163" t="s">
         <v>85</v>
       </c>
@@ -8118,7 +8112,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="164" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B164" t="s">
         <v>85</v>
       </c>
@@ -8207,7 +8201,7 @@
         <v>226.5</v>
       </c>
       <c r="F166" s="3">
-        <v>258.7</v>
+        <v>210.7</v>
       </c>
       <c r="L166" s="4"/>
       <c r="M166" s="4"/>
@@ -8227,7 +8221,7 @@
         <v>100.7</v>
       </c>
       <c r="AA166" s="4">
-        <v>158</v>
+        <v>110</v>
       </c>
       <c r="AB166" s="4"/>
       <c r="AC166" s="4"/>
@@ -8235,7 +8229,7 @@
       <c r="AE166" s="4"/>
       <c r="AF166" s="4"/>
     </row>
-    <row r="167" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B167" t="s">
         <v>95</v>
       </c>
@@ -8267,7 +8261,7 @@
       <c r="AE167" s="4"/>
       <c r="AF167" s="4"/>
     </row>
-    <row r="168" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B168" t="s">
         <v>95</v>
       </c>
@@ -8281,7 +8275,7 @@
         <v>1566.27</v>
       </c>
       <c r="F168" s="3">
-        <v>332</v>
+        <v>401</v>
       </c>
       <c r="L168" s="4"/>
       <c r="M168" s="4"/>
@@ -8301,7 +8295,7 @@
         <v>42</v>
       </c>
       <c r="AA168" s="4">
-        <v>290</v>
+        <v>359</v>
       </c>
       <c r="AB168" s="4"/>
       <c r="AC168" s="4"/>
@@ -8309,7 +8303,7 @@
       <c r="AE168" s="4"/>
       <c r="AF168" s="4"/>
     </row>
-    <row r="169" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B169" t="s">
         <v>91</v>
       </c>
@@ -8344,7 +8338,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="170" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B170" t="s">
         <v>91</v>
       </c>
@@ -8391,7 +8385,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="171" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B171" t="s">
         <v>42</v>
       </c>
@@ -8429,7 +8423,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="172" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B172" t="s">
         <v>42</v>
       </c>
@@ -8464,7 +8458,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="173" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B173" t="s">
         <v>68</v>
       </c>
@@ -8499,7 +8493,7 @@
       <c r="AE173" s="4"/>
       <c r="AF173" s="4"/>
     </row>
-    <row r="174" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B174" t="s">
         <v>68</v>
       </c>
@@ -8534,7 +8528,7 @@
       <c r="AE174" s="4"/>
       <c r="AF174" s="4"/>
     </row>
-    <row r="175" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B175" t="s">
         <v>98</v>
       </c>
@@ -8580,7 +8574,7 @@
       <c r="AE175" s="4"/>
       <c r="AF175" s="4"/>
     </row>
-    <row r="176" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B176" t="s">
         <v>98</v>
       </c>
@@ -8624,7 +8618,7 @@
       <c r="AE176" s="4"/>
       <c r="AF176" s="4"/>
     </row>
-    <row r="177" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B177" t="s">
         <v>100</v>
       </c>
@@ -8659,7 +8653,7 @@
       <c r="AE177" s="4"/>
       <c r="AF177" s="4"/>
     </row>
-    <row r="178" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B178" t="s">
         <v>100</v>
       </c>
@@ -8694,7 +8688,7 @@
       <c r="AE178" s="4"/>
       <c r="AF178" s="4"/>
     </row>
-    <row r="179" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B179" t="s">
         <v>102</v>
       </c>
@@ -8729,7 +8723,7 @@
       <c r="AE179" s="4"/>
       <c r="AF179" s="4"/>
     </row>
-    <row r="180" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B180" t="s">
         <v>102</v>
       </c>
@@ -8764,7 +8758,7 @@
       <c r="AE180" s="4"/>
       <c r="AF180" s="4"/>
     </row>
-    <row r="181" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B181" t="s">
         <v>104</v>
       </c>
@@ -8799,7 +8793,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="182" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B182" t="s">
         <v>104</v>
       </c>
@@ -8837,7 +8831,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="183" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B183" t="s">
         <v>90</v>
       </c>
@@ -8872,7 +8866,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="184" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B184" t="s">
         <v>90</v>
       </c>
@@ -8907,7 +8901,7 @@
       <c r="AE184" s="4"/>
       <c r="AF184" s="4"/>
     </row>
-    <row r="185" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B185" t="s">
         <v>78</v>
       </c>
@@ -8945,7 +8939,7 @@
       <c r="AE185" s="4"/>
       <c r="AF185" s="4"/>
     </row>
-    <row r="186" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B186" t="s">
         <v>78</v>
       </c>
@@ -8980,7 +8974,7 @@
       <c r="AE186" s="4"/>
       <c r="AF186" s="4"/>
     </row>
-    <row r="187" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B187" t="s">
         <v>44</v>
       </c>
@@ -9020,7 +9014,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="188" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B188" t="s">
         <v>44</v>
       </c>
@@ -9058,7 +9052,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="189" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B189" t="s">
         <v>45</v>
       </c>
@@ -9090,7 +9084,7 @@
       <c r="AE189" s="4"/>
       <c r="AF189" s="4"/>
     </row>
-    <row r="190" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B190" t="s">
         <v>45</v>
       </c>
@@ -9125,7 +9119,7 @@
       <c r="AE190" s="4"/>
       <c r="AF190" s="4"/>
     </row>
-    <row r="191" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B191" t="s">
         <v>54</v>
       </c>
@@ -9157,7 +9151,7 @@
       <c r="AE191" s="4"/>
       <c r="AF191" s="4"/>
     </row>
-    <row r="192" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B192" t="s">
         <v>54</v>
       </c>
@@ -9193,7 +9187,7 @@
       <c r="AE192" s="4"/>
       <c r="AF192" s="4"/>
     </row>
-    <row r="193" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B193" t="s">
         <v>43</v>
       </c>
@@ -9225,7 +9219,7 @@
       <c r="AE193" s="4"/>
       <c r="AF193" s="4"/>
     </row>
-    <row r="194" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B194" t="s">
         <v>43</v>
       </c>
@@ -9260,7 +9254,7 @@
       <c r="AE194" s="4"/>
       <c r="AF194" s="4"/>
     </row>
-    <row r="195" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B195" t="s">
         <v>92</v>
       </c>
@@ -9298,7 +9292,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="196" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B196" t="s">
         <v>92</v>
       </c>
@@ -9336,7 +9330,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="197" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B197" t="s">
         <v>46</v>
       </c>
@@ -9371,7 +9365,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="198" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B198" t="s">
         <v>46</v>
       </c>
@@ -9409,7 +9403,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="199" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B199" t="s">
         <v>41</v>
       </c>
@@ -9447,7 +9441,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="200" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B200" t="s">
         <v>41</v>
       </c>
@@ -9485,7 +9479,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="201" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B201" t="s">
         <v>61</v>
       </c>
@@ -9520,7 +9514,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="202" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B202" t="s">
         <v>61</v>
       </c>
@@ -9558,7 +9552,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="203" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B203" t="s">
         <v>96</v>
       </c>
@@ -9593,7 +9587,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="204" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B204" t="s">
         <v>96</v>
       </c>
@@ -9636,7 +9630,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="205" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B205" t="s">
         <v>69</v>
       </c>
@@ -9680,7 +9674,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="206" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B206" t="s">
         <v>69</v>
       </c>
@@ -9727,7 +9721,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="207" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B207" t="s">
         <v>72</v>
       </c>
@@ -9765,7 +9759,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="208" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B208" t="s">
         <v>72</v>
       </c>
@@ -9779,7 +9773,7 @@
         <v>382.5</v>
       </c>
       <c r="F208" s="3">
-        <v>42</v>
+        <v>68</v>
       </c>
       <c r="L208" s="4"/>
       <c r="M208" s="4"/>
@@ -9797,7 +9791,7 @@
       <c r="Y208" s="4"/>
       <c r="Z208" s="9"/>
       <c r="AA208" s="4">
-        <v>42</v>
+        <v>68</v>
       </c>
       <c r="AB208" s="4"/>
       <c r="AC208" s="4"/>
@@ -9808,7 +9802,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="209" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B209" t="s">
         <v>84</v>
       </c>
@@ -9849,7 +9843,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="210" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B210" t="s">
         <v>84</v>
       </c>
@@ -9887,7 +9881,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="211" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B211" t="s">
         <v>94</v>
       </c>
@@ -9922,7 +9916,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="212" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B212" t="s">
         <v>94</v>
       </c>
@@ -9960,7 +9954,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="213" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B213" t="s">
         <v>75</v>
       </c>
@@ -10001,7 +9995,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="214" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B214" t="s">
         <v>75</v>
       </c>
@@ -10039,7 +10033,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="215" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B215" t="s">
         <v>73</v>
       </c>
@@ -10077,7 +10071,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="216" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B216" t="s">
         <v>73</v>
       </c>
@@ -10115,7 +10109,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="217" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B217" t="s">
         <v>39</v>
       </c>
@@ -10156,7 +10150,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="218" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B218" t="s">
         <v>39</v>
       </c>

</xml_diff>

<commit_message>
Atualiza PDS e planilhas de 2026-07-21
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA143249-3D47-4B4D-89D2-DB81D518D575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A6D93DF-D2A3-4536-BFA7-4CF39D87C8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="665" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="124">
   <si>
     <t>Data</t>
   </si>
@@ -316,9 +316,6 @@
   </si>
   <si>
     <t xml:space="preserve">RCE RUA JOSÉ MILITÃO </t>
-  </si>
-  <si>
-    <t>rede existente</t>
   </si>
   <si>
     <t>RCE VIELA DA RUA INÊS SABINO</t>
@@ -799,7 +796,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tb_base_dash_extensao" displayName="tb_base_dash_extensao" ref="B1:AF218">
-  <autoFilter ref="B1:AF218" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <autoFilter ref="B1:AF218" xr:uid="{00000000-0009-0000-0100-000001000000}">
+    <filterColumn colId="25">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:AF218">
     <sortCondition ref="B1:B218"/>
   </sortState>
@@ -1253,7 +1256,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B2" s="3" t="s">
         <v>64</v>
       </c>
@@ -1310,7 +1313,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B3" s="3" t="s">
         <v>64</v>
       </c>
@@ -1353,7 +1356,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>64</v>
       </c>
@@ -1399,7 +1402,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B5" s="3" t="s">
         <v>64</v>
       </c>
@@ -1442,7 +1445,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
         <v>64</v>
       </c>
@@ -1488,7 +1491,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B7" s="3" t="s">
         <v>64</v>
       </c>
@@ -1531,7 +1534,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B8" s="3" t="s">
         <v>63</v>
       </c>
@@ -1579,7 +1582,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B9" s="3" t="s">
         <v>63</v>
       </c>
@@ -1622,7 +1625,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B10" s="3" t="s">
         <v>63</v>
       </c>
@@ -1667,7 +1670,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B11" s="3" t="s">
         <v>63</v>
       </c>
@@ -1705,7 +1708,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B12" s="3" t="s">
         <v>63</v>
       </c>
@@ -1748,7 +1751,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B13" s="3" t="s">
         <v>63</v>
       </c>
@@ -1786,7 +1789,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
         <v>63</v>
       </c>
@@ -1831,7 +1834,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B15" s="3" t="s">
         <v>63</v>
       </c>
@@ -1869,7 +1872,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:33" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
         <v>63</v>
       </c>
@@ -1914,7 +1917,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B17" s="3" t="s">
         <v>63</v>
       </c>
@@ -1952,7 +1955,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="18" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B18" s="3" t="s">
         <v>63</v>
       </c>
@@ -1995,7 +1998,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B19" s="3" t="s">
         <v>63</v>
       </c>
@@ -2033,7 +2036,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B20" s="3" t="s">
         <v>63</v>
       </c>
@@ -2076,7 +2079,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="21" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B21" s="3" t="s">
         <v>63</v>
       </c>
@@ -2114,7 +2117,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B22" s="3" t="s">
         <v>63</v>
       </c>
@@ -2157,7 +2160,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B23" s="3" t="s">
         <v>63</v>
       </c>
@@ -2195,7 +2198,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="24" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B24" s="3" t="s">
         <v>63</v>
       </c>
@@ -2237,10 +2240,10 @@
       <c r="AE24" s="4"/>
       <c r="AF24" s="4"/>
       <c r="AG24" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="25" spans="2:33" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="25" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B25" s="3" t="s">
         <v>63</v>
       </c>
@@ -2278,10 +2281,10 @@
       <c r="AE25" s="4"/>
       <c r="AF25" s="4"/>
       <c r="AG25" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="26" spans="2:33" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="26" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B26" s="3" t="s">
         <v>62</v>
       </c>
@@ -2322,8 +2325,11 @@
       <c r="AD26" s="4"/>
       <c r="AE26" s="4"/>
       <c r="AF26" s="4"/>
-    </row>
-    <row r="27" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG26" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="27" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B27" s="3" t="s">
         <v>62</v>
       </c>
@@ -2364,8 +2370,11 @@
       <c r="AD27" s="4"/>
       <c r="AE27" s="4"/>
       <c r="AF27" s="4"/>
-    </row>
-    <row r="28" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG27" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="28" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B28" s="3" t="s">
         <v>62</v>
       </c>
@@ -2404,8 +2413,11 @@
       <c r="AD28" s="4"/>
       <c r="AE28" s="4"/>
       <c r="AF28" s="4"/>
-    </row>
-    <row r="29" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG28" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="29" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
         <v>62</v>
       </c>
@@ -2439,8 +2451,11 @@
       <c r="AD29" s="4"/>
       <c r="AE29" s="4"/>
       <c r="AF29" s="4"/>
-    </row>
-    <row r="30" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG29" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="30" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B30" s="3" t="s">
         <v>62</v>
       </c>
@@ -2476,8 +2491,11 @@
       <c r="AD30" s="4"/>
       <c r="AE30" s="4"/>
       <c r="AF30" s="4"/>
-    </row>
-    <row r="31" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG30" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="31" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B31" s="3" t="s">
         <v>62</v>
       </c>
@@ -2511,8 +2529,11 @@
       <c r="AD31" s="4"/>
       <c r="AE31" s="4"/>
       <c r="AF31" s="4"/>
-    </row>
-    <row r="32" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG31" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="32" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B32" s="3" t="s">
         <v>62</v>
       </c>
@@ -2552,7 +2573,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="33" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B33" s="3" t="s">
         <v>62</v>
       </c>
@@ -2587,10 +2608,10 @@
       <c r="AE33" s="4"/>
       <c r="AF33" s="4"/>
       <c r="AG33" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="34" spans="2:33" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="34" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B34" s="3" t="s">
         <v>62</v>
       </c>
@@ -2629,8 +2650,11 @@
       <c r="AD34" s="4"/>
       <c r="AE34" s="4"/>
       <c r="AF34" s="4"/>
-    </row>
-    <row r="35" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG34" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="35" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B35" s="3" t="s">
         <v>62</v>
       </c>
@@ -2664,8 +2688,11 @@
       <c r="AD35" s="4"/>
       <c r="AE35" s="4"/>
       <c r="AF35" s="4"/>
-    </row>
-    <row r="36" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG35" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="36" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B36" s="3" t="s">
         <v>62</v>
       </c>
@@ -2701,8 +2728,11 @@
       <c r="AD36" s="4"/>
       <c r="AE36" s="4"/>
       <c r="AF36" s="4"/>
-    </row>
-    <row r="37" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG36" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B37" s="3" t="s">
         <v>62</v>
       </c>
@@ -2736,8 +2766,11 @@
       <c r="AD37" s="4"/>
       <c r="AE37" s="4"/>
       <c r="AF37" s="4"/>
-    </row>
-    <row r="38" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG37" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="38" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B38" s="3" t="s">
         <v>62</v>
       </c>
@@ -2774,10 +2807,10 @@
       <c r="AE38" s="4"/>
       <c r="AF38" s="4"/>
       <c r="AG38" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="39" spans="2:33" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="39" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B39" s="3" t="s">
         <v>62</v>
       </c>
@@ -2811,8 +2844,11 @@
       <c r="AD39" s="4"/>
       <c r="AE39" s="4"/>
       <c r="AF39" s="4"/>
-    </row>
-    <row r="40" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG39" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="40" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B40" s="3" t="s">
         <v>62</v>
       </c>
@@ -2848,8 +2884,11 @@
       <c r="AD40" s="4"/>
       <c r="AE40" s="4"/>
       <c r="AF40" s="4"/>
-    </row>
-    <row r="41" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG40" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="41" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B41" s="3" t="s">
         <v>62</v>
       </c>
@@ -2883,8 +2922,11 @@
       <c r="AD41" s="4"/>
       <c r="AE41" s="4"/>
       <c r="AF41" s="4"/>
-    </row>
-    <row r="42" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG41" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="42" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B42" s="3" t="s">
         <v>62</v>
       </c>
@@ -2920,8 +2962,11 @@
       <c r="AD42" s="4"/>
       <c r="AE42" s="4"/>
       <c r="AF42" s="4"/>
-    </row>
-    <row r="43" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG42" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="43" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B43" s="3" t="s">
         <v>62</v>
       </c>
@@ -2955,8 +3000,11 @@
       <c r="AD43" s="4"/>
       <c r="AE43" s="4"/>
       <c r="AF43" s="4"/>
-    </row>
-    <row r="44" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG43" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="44" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B44" s="3" t="s">
         <v>62</v>
       </c>
@@ -2995,8 +3043,11 @@
       <c r="AD44" s="4"/>
       <c r="AE44" s="4"/>
       <c r="AF44" s="4"/>
-    </row>
-    <row r="45" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG44" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="45" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B45" s="3" t="s">
         <v>62</v>
       </c>
@@ -3030,8 +3081,11 @@
       <c r="AD45" s="4"/>
       <c r="AE45" s="4"/>
       <c r="AF45" s="4"/>
-    </row>
-    <row r="46" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG45" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="46" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B46" s="3" t="s">
         <v>62</v>
       </c>
@@ -3072,8 +3126,11 @@
       <c r="AD46" s="4"/>
       <c r="AE46" s="4"/>
       <c r="AF46" s="4"/>
-    </row>
-    <row r="47" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG46" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="47" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B47" s="3" t="s">
         <v>62</v>
       </c>
@@ -3107,8 +3164,11 @@
       <c r="AD47" s="4"/>
       <c r="AE47" s="4"/>
       <c r="AF47" s="4"/>
-    </row>
-    <row r="48" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG47" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="48" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B48" s="3" t="s">
         <v>62</v>
       </c>
@@ -3149,8 +3209,11 @@
       <c r="AD48" s="4"/>
       <c r="AE48" s="4"/>
       <c r="AF48" s="4"/>
-    </row>
-    <row r="49" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG48" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="49" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B49" s="3" t="s">
         <v>62</v>
       </c>
@@ -3184,8 +3247,11 @@
       <c r="AD49" s="4"/>
       <c r="AE49" s="4"/>
       <c r="AF49" s="4"/>
-    </row>
-    <row r="50" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG49" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="50" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B50" s="3" t="s">
         <v>62</v>
       </c>
@@ -3224,8 +3290,11 @@
       <c r="AD50" s="4"/>
       <c r="AE50" s="4"/>
       <c r="AF50" s="4"/>
-    </row>
-    <row r="51" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG50" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="51" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B51" s="3" t="s">
         <v>62</v>
       </c>
@@ -3259,8 +3328,11 @@
       <c r="AD51" s="4"/>
       <c r="AE51" s="4"/>
       <c r="AF51" s="4"/>
-    </row>
-    <row r="52" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG51" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="52" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B52" s="3" t="s">
         <v>62</v>
       </c>
@@ -3299,8 +3371,11 @@
       <c r="AD52" s="4"/>
       <c r="AE52" s="4"/>
       <c r="AF52" s="4"/>
-    </row>
-    <row r="53" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG52" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="53" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B53" s="3" t="s">
         <v>62</v>
       </c>
@@ -3334,8 +3409,11 @@
       <c r="AD53" s="4"/>
       <c r="AE53" s="4"/>
       <c r="AF53" s="4"/>
-    </row>
-    <row r="54" spans="2:33" x14ac:dyDescent="0.3">
+      <c r="AG53" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="54" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B54" s="3" t="s">
         <v>62</v>
       </c>
@@ -3377,10 +3455,10 @@
       <c r="AE54" s="4"/>
       <c r="AF54" s="4"/>
       <c r="AG54" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="55" spans="2:33" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="55" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B55" s="3" t="s">
         <v>62</v>
       </c>
@@ -3418,7 +3496,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="56" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B56" s="3" t="s">
         <v>62</v>
       </c>
@@ -3464,7 +3542,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="57" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B57" s="3" t="s">
         <v>62</v>
       </c>
@@ -3507,12 +3585,12 @@
         <v>35</v>
       </c>
     </row>
-    <row r="58" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B58" s="3" t="s">
         <v>62</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D58" t="s">
         <v>34</v>
@@ -3550,12 +3628,12 @@
         <v>35</v>
       </c>
     </row>
-    <row r="59" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B59" s="3" t="s">
         <v>62</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D59" t="s">
         <v>36</v>
@@ -3588,7 +3666,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="60" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B60" s="3" t="s">
         <v>58</v>
       </c>
@@ -3653,7 +3731,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="61" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B61" s="3" t="s">
         <v>58</v>
       </c>
@@ -3696,7 +3774,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="62" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B62" s="3" t="s">
         <v>58</v>
       </c>
@@ -3752,7 +3830,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="63" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B63" s="3" t="s">
         <v>58</v>
       </c>
@@ -3794,7 +3872,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="64" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B64" s="3" t="s">
         <v>58</v>
       </c>
@@ -3852,7 +3930,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="65" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B65" s="3" t="s">
         <v>58</v>
       </c>
@@ -3896,7 +3974,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="66" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B66" s="3" t="s">
         <v>59</v>
       </c>
@@ -3943,7 +4021,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="67" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B67" s="3" t="s">
         <v>59</v>
       </c>
@@ -3988,7 +4066,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="68" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B68" s="3" t="s">
         <v>59</v>
       </c>
@@ -4035,7 +4113,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="69" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B69" s="3" t="s">
         <v>59</v>
       </c>
@@ -4079,7 +4157,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="70" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B70" s="3" t="s">
         <v>33</v>
       </c>
@@ -4125,7 +4203,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="71" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B71" s="3" t="s">
         <v>33</v>
       </c>
@@ -4168,7 +4246,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="72" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B72" s="3" t="s">
         <v>33</v>
       </c>
@@ -4213,7 +4291,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="73" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B73" s="3" t="s">
         <v>33</v>
       </c>
@@ -4256,7 +4334,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="74" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B74" s="3" t="s">
         <v>33</v>
       </c>
@@ -4299,7 +4377,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="75" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B75" s="3" t="s">
         <v>33</v>
       </c>
@@ -4342,7 +4420,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="76" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B76" s="3" t="s">
         <v>33</v>
       </c>
@@ -4390,7 +4468,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="77" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B77" s="3" t="s">
         <v>33</v>
       </c>
@@ -4434,7 +4512,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="78" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B78" s="3" t="s">
         <v>38</v>
       </c>
@@ -4489,7 +4567,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="79" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B79" s="3" t="s">
         <v>38</v>
       </c>
@@ -4532,7 +4610,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="80" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B80" s="3" t="s">
         <v>38</v>
       </c>
@@ -4581,7 +4659,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="81" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B81" s="3" t="s">
         <v>38</v>
       </c>
@@ -4624,7 +4702,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="82" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B82" s="3" t="s">
         <v>60</v>
       </c>
@@ -4673,7 +4751,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="83" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B83" s="3" t="s">
         <v>60</v>
       </c>
@@ -4716,7 +4794,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="84" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B84" s="3" t="s">
         <v>57</v>
       </c>
@@ -4772,7 +4850,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="85" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B85" s="3" t="s">
         <v>57</v>
       </c>
@@ -4816,7 +4894,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="86" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B86" s="3" t="s">
         <v>57</v>
       </c>
@@ -4866,7 +4944,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="87" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B87" s="3" t="s">
         <v>57</v>
       </c>
@@ -4910,7 +4988,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="88" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B88" s="3" t="s">
         <v>57</v>
       </c>
@@ -4962,7 +5040,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="89" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B89" s="3" t="s">
         <v>57</v>
       </c>
@@ -5006,7 +5084,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="90" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B90" t="s">
         <v>52</v>
       </c>
@@ -5040,11 +5118,8 @@
       <c r="AD90" s="4"/>
       <c r="AE90" s="4"/>
       <c r="AF90" s="4"/>
-      <c r="AG90" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="91" spans="2:33" x14ac:dyDescent="0.3">
+    </row>
+    <row r="91" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B91" t="s">
         <v>52</v>
       </c>
@@ -5078,11 +5153,8 @@
       <c r="AD91" s="4"/>
       <c r="AE91" s="4"/>
       <c r="AF91" s="4"/>
-      <c r="AG91" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="92" spans="2:33" x14ac:dyDescent="0.3">
+    </row>
+    <row r="92" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B92" s="3" t="s">
         <v>56</v>
       </c>
@@ -5134,7 +5206,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="93" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B93" s="3" t="s">
         <v>56</v>
       </c>
@@ -5176,7 +5248,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="94" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B94" s="3" t="s">
         <v>56</v>
       </c>
@@ -5228,7 +5300,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="95" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B95" s="3" t="s">
         <v>56</v>
       </c>
@@ -5270,7 +5342,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="96" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B96" s="3" t="s">
         <v>56</v>
       </c>
@@ -5322,7 +5394,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="97" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B97" s="3" t="s">
         <v>56</v>
       </c>
@@ -5366,7 +5438,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="98" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B98" s="3" t="s">
         <v>56</v>
       </c>
@@ -5413,7 +5485,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="99" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B99" s="3" t="s">
         <v>56</v>
       </c>
@@ -5457,7 +5529,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="100" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B100" s="3" t="s">
         <v>55</v>
       </c>
@@ -5504,7 +5576,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="101" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B101" s="3" t="s">
         <v>37</v>
       </c>
@@ -5561,7 +5633,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="102" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B102" s="3" t="s">
         <v>37</v>
       </c>
@@ -5599,7 +5671,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="103" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B103" s="3" t="s">
         <v>37</v>
       </c>
@@ -5650,7 +5722,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="104" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B104" s="3" t="s">
         <v>37</v>
       </c>
@@ -5691,7 +5763,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="105" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B105" s="3" t="s">
         <v>37</v>
       </c>
@@ -5742,7 +5814,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="106" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:33" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B106" s="3" t="s">
         <v>37</v>
       </c>
@@ -5785,7 +5857,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="107" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B107" s="3" t="s">
         <v>37</v>
       </c>
@@ -5838,7 +5910,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="108" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B108" s="3" t="s">
         <v>37</v>
       </c>
@@ -5876,7 +5948,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="109" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B109" s="3" t="s">
         <v>37</v>
       </c>
@@ -5925,7 +5997,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="110" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B110" s="3" t="s">
         <v>37</v>
       </c>
@@ -5974,7 +6046,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="111" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B111" t="s">
         <v>89</v>
       </c>
@@ -6015,10 +6087,10 @@
       <c r="AE111" s="4"/>
       <c r="AF111" s="4"/>
       <c r="AG111" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="112" spans="2:33" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="112" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B112" t="s">
         <v>89</v>
       </c>
@@ -6053,10 +6125,10 @@
       <c r="AE112" s="4"/>
       <c r="AF112" s="4"/>
       <c r="AG112" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="113" spans="2:33" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="113" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B113" s="3" t="s">
         <v>77</v>
       </c>
@@ -6102,7 +6174,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="114" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B114" s="3" t="s">
         <v>77</v>
       </c>
@@ -6140,7 +6212,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="115" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B115" s="3" t="s">
         <v>77</v>
       </c>
@@ -6189,7 +6261,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="116" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B116" s="3" t="s">
         <v>77</v>
       </c>
@@ -6232,7 +6304,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="117" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B117" s="3" t="s">
         <v>74</v>
       </c>
@@ -6293,7 +6365,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="118" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B118" s="3" t="s">
         <v>74</v>
       </c>
@@ -6342,7 +6414,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="119" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B119" s="3" t="s">
         <v>74</v>
       </c>
@@ -6401,7 +6473,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="120" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B120" s="3" t="s">
         <v>74</v>
       </c>
@@ -6447,7 +6519,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="121" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B121" s="3" t="s">
         <v>74</v>
       </c>
@@ -6496,7 +6568,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="122" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="122" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B122" s="3" t="s">
         <v>74</v>
       </c>
@@ -6539,7 +6611,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="123" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B123" t="s">
         <v>50</v>
       </c>
@@ -6573,11 +6645,8 @@
       <c r="AD123" s="4"/>
       <c r="AE123" s="4"/>
       <c r="AF123" s="4"/>
-      <c r="AG123" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="124" spans="2:33" x14ac:dyDescent="0.3">
+    </row>
+    <row r="124" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B124" t="s">
         <v>50</v>
       </c>
@@ -6608,11 +6677,8 @@
       <c r="AD124" s="4"/>
       <c r="AE124" s="4"/>
       <c r="AF124" s="4"/>
-      <c r="AG124" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="125" spans="2:33" x14ac:dyDescent="0.3">
+    </row>
+    <row r="125" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B125" t="s">
         <v>53</v>
       </c>
@@ -6646,11 +6712,8 @@
       <c r="AD125" s="4"/>
       <c r="AE125" s="4"/>
       <c r="AF125" s="4"/>
-      <c r="AG125" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="126" spans="2:33" x14ac:dyDescent="0.3">
+    </row>
+    <row r="126" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B126" t="s">
         <v>53</v>
       </c>
@@ -6684,11 +6747,8 @@
       <c r="AD126" s="4"/>
       <c r="AE126" s="4"/>
       <c r="AF126" s="4"/>
-      <c r="AG126" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="127" spans="2:33" x14ac:dyDescent="0.3">
+    </row>
+    <row r="127" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B127" t="s">
         <v>48</v>
       </c>
@@ -6722,11 +6782,8 @@
       <c r="AD127" s="4"/>
       <c r="AE127" s="4"/>
       <c r="AF127" s="4"/>
-      <c r="AG127" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="128" spans="2:33" x14ac:dyDescent="0.3">
+    </row>
+    <row r="128" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B128" t="s">
         <v>48</v>
       </c>
@@ -6757,11 +6814,8 @@
       <c r="AD128" s="4"/>
       <c r="AE128" s="4"/>
       <c r="AF128" s="4"/>
-      <c r="AG128" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="129" spans="2:33" x14ac:dyDescent="0.3">
+    </row>
+    <row r="129" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B129" t="s">
         <v>70</v>
       </c>
@@ -6792,11 +6846,8 @@
       <c r="AD129" s="4"/>
       <c r="AE129" s="4"/>
       <c r="AF129" s="4"/>
-      <c r="AG129" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="130" spans="2:33" x14ac:dyDescent="0.3">
+    </row>
+    <row r="130" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B130" t="s">
         <v>70</v>
       </c>
@@ -6830,11 +6881,8 @@
       <c r="AD130" s="4"/>
       <c r="AE130" s="4"/>
       <c r="AF130" s="4"/>
-      <c r="AG130" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="131" spans="2:33" x14ac:dyDescent="0.3">
+    </row>
+    <row r="131" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B131" s="3" t="s">
         <v>82</v>
       </c>
@@ -6883,7 +6931,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="132" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="132" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B132" s="3" t="s">
         <v>82</v>
       </c>
@@ -6927,8 +6975,8 @@
         <v>35</v>
       </c>
     </row>
-    <row r="133" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B133" t="s">
+    <row r="133" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B133" s="3" t="s">
         <v>71</v>
       </c>
       <c r="C133">
@@ -6965,8 +7013,8 @@
         <v>35</v>
       </c>
     </row>
-    <row r="134" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B134" t="s">
+    <row r="134" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B134" s="3" t="s">
         <v>71</v>
       </c>
       <c r="C134">
@@ -7008,8 +7056,8 @@
         <v>35</v>
       </c>
     </row>
-    <row r="135" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B135" t="s">
+    <row r="135" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B135" s="3" t="s">
         <v>80</v>
       </c>
       <c r="C135">
@@ -7049,8 +7097,8 @@
         <v>35</v>
       </c>
     </row>
-    <row r="136" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B136" t="s">
+    <row r="136" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B136" s="3" t="s">
         <v>80</v>
       </c>
       <c r="C136">
@@ -7087,8 +7135,8 @@
         <v>35</v>
       </c>
     </row>
-    <row r="137" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B137" t="s">
+    <row r="137" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B137" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C137">
@@ -7121,12 +7169,9 @@
       <c r="AD137" s="4"/>
       <c r="AE137" s="4"/>
       <c r="AF137" s="4"/>
-      <c r="AG137" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="138" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B138" t="s">
+    </row>
+    <row r="138" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B138" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C138">
@@ -7159,12 +7204,9 @@
       <c r="AD138" s="4"/>
       <c r="AE138" s="4"/>
       <c r="AF138" s="4"/>
-      <c r="AG138" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="139" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B139" t="s">
+    </row>
+    <row r="139" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B139" s="3" t="s">
         <v>49</v>
       </c>
       <c r="C139">
@@ -7197,12 +7239,9 @@
       <c r="AD139" s="4"/>
       <c r="AE139" s="4"/>
       <c r="AF139" s="4"/>
-      <c r="AG139" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="140" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B140" t="s">
+    </row>
+    <row r="140" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B140" s="3" t="s">
         <v>49</v>
       </c>
       <c r="C140">
@@ -7232,12 +7271,9 @@
       <c r="AD140" s="4"/>
       <c r="AE140" s="4"/>
       <c r="AF140" s="4"/>
-      <c r="AG140" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="141" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B141" t="s">
+    </row>
+    <row r="141" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B141" s="3" t="s">
         <v>81</v>
       </c>
       <c r="C141">
@@ -7267,12 +7303,9 @@
       <c r="AD141" s="4"/>
       <c r="AE141" s="4"/>
       <c r="AF141" s="4"/>
-      <c r="AG141" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="142" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B142" t="s">
+    </row>
+    <row r="142" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B142" s="3" t="s">
         <v>81</v>
       </c>
       <c r="C142">
@@ -7305,12 +7338,9 @@
       <c r="AD142" s="4"/>
       <c r="AE142" s="4"/>
       <c r="AF142" s="4"/>
-      <c r="AG142" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="143" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B143" t="s">
+    </row>
+    <row r="143" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B143" s="3" t="s">
         <v>47</v>
       </c>
       <c r="C143" s="1">
@@ -7345,7 +7375,7 @@
       </c>
     </row>
     <row r="144" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B144" t="s">
+      <c r="B144" s="3" t="s">
         <v>47</v>
       </c>
       <c r="C144" s="1">
@@ -7389,8 +7419,8 @@
         <v>35</v>
       </c>
     </row>
-    <row r="145" spans="2:38" x14ac:dyDescent="0.3">
-      <c r="B145" t="s">
+    <row r="145" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B145" s="3" t="s">
         <v>65</v>
       </c>
       <c r="C145">
@@ -7434,9 +7464,12 @@
       <c r="AD145" s="4"/>
       <c r="AE145" s="4"/>
       <c r="AF145" s="4"/>
-    </row>
-    <row r="146" spans="2:38" x14ac:dyDescent="0.3">
-      <c r="B146" t="s">
+      <c r="AG145" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="146" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B146" s="3" t="s">
         <v>65</v>
       </c>
       <c r="C146">
@@ -7472,9 +7505,12 @@
       <c r="AD146" s="4"/>
       <c r="AE146" s="4"/>
       <c r="AF146" s="4"/>
-    </row>
-    <row r="147" spans="2:38" x14ac:dyDescent="0.3">
-      <c r="B147" t="s">
+      <c r="AG146" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="147" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B147" s="3" t="s">
         <v>65</v>
       </c>
       <c r="C147">
@@ -7519,9 +7555,12 @@
       <c r="AD147" s="4"/>
       <c r="AE147" s="4"/>
       <c r="AF147" s="4"/>
-    </row>
-    <row r="148" spans="2:38" x14ac:dyDescent="0.3">
-      <c r="B148" t="s">
+      <c r="AG147" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="148" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B148" s="3" t="s">
         <v>65</v>
       </c>
       <c r="C148">
@@ -7561,9 +7600,12 @@
       <c r="AD148" s="4"/>
       <c r="AE148" s="4"/>
       <c r="AF148" s="4"/>
-    </row>
-    <row r="149" spans="2:38" x14ac:dyDescent="0.3">
-      <c r="B149" t="s">
+      <c r="AG148" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="149" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B149" s="3" t="s">
         <v>79</v>
       </c>
       <c r="C149">
@@ -7594,8 +7636,8 @@
       <c r="AE149" s="4"/>
       <c r="AF149" s="4"/>
     </row>
-    <row r="150" spans="2:38" x14ac:dyDescent="0.3">
-      <c r="B150" t="s">
+    <row r="150" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B150" s="3" t="s">
         <v>79</v>
       </c>
       <c r="C150">
@@ -7628,11 +7670,8 @@
       <c r="AD150" s="4"/>
       <c r="AE150" s="4"/>
       <c r="AF150" s="4"/>
-      <c r="AG150" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="151" spans="2:38" x14ac:dyDescent="0.3">
+    </row>
+    <row r="151" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
       <c r="B151" s="3" t="s">
         <v>66</v>
       </c>
@@ -7675,7 +7714,7 @@
       <c r="AE151" s="4"/>
       <c r="AF151" s="4"/>
     </row>
-    <row r="152" spans="2:38" x14ac:dyDescent="0.3">
+    <row r="152" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
       <c r="B152" s="3" t="s">
         <v>66</v>
       </c>
@@ -7710,8 +7749,8 @@
       <c r="AE152" s="4"/>
       <c r="AF152" s="4"/>
     </row>
-    <row r="153" spans="2:38" x14ac:dyDescent="0.3">
-      <c r="B153" t="s">
+    <row r="153" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B153" s="3" t="s">
         <v>67</v>
       </c>
       <c r="C153">
@@ -7748,8 +7787,8 @@
       <c r="AE153" s="4"/>
       <c r="AF153" s="4"/>
     </row>
-    <row r="154" spans="2:38" x14ac:dyDescent="0.3">
-      <c r="B154" t="s">
+    <row r="154" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B154" s="3" t="s">
         <v>67</v>
       </c>
       <c r="C154">
@@ -7783,8 +7822,8 @@
       <c r="AE154" s="4"/>
       <c r="AF154" s="4"/>
     </row>
-    <row r="155" spans="2:38" x14ac:dyDescent="0.3">
-      <c r="B155" t="s">
+    <row r="155" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B155" s="3" t="s">
         <v>86</v>
       </c>
       <c r="C155">
@@ -7818,8 +7857,8 @@
         <v>1746.61</v>
       </c>
     </row>
-    <row r="156" spans="2:38" x14ac:dyDescent="0.3">
-      <c r="B156" t="s">
+    <row r="156" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B156" s="3" t="s">
         <v>86</v>
       </c>
       <c r="C156">
@@ -7856,8 +7895,8 @@
         <v>1471.49</v>
       </c>
     </row>
-    <row r="157" spans="2:38" x14ac:dyDescent="0.3">
-      <c r="B157" t="s">
+    <row r="157" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B157" s="3" t="s">
         <v>87</v>
       </c>
       <c r="C157">
@@ -7892,8 +7931,8 @@
         <v>275.11999999999989</v>
       </c>
     </row>
-    <row r="158" spans="2:38" x14ac:dyDescent="0.3">
-      <c r="B158" t="s">
+    <row r="158" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B158" s="3" t="s">
         <v>87</v>
       </c>
       <c r="C158">
@@ -7927,8 +7966,8 @@
       <c r="AE158" s="4"/>
       <c r="AF158" s="4"/>
     </row>
-    <row r="159" spans="2:38" x14ac:dyDescent="0.3">
-      <c r="B159" t="s">
+    <row r="159" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B159" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C159">
@@ -7958,12 +7997,9 @@
       <c r="AD159" s="4"/>
       <c r="AE159" s="4"/>
       <c r="AF159" s="4"/>
-      <c r="AG159" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="160" spans="2:38" x14ac:dyDescent="0.3">
-      <c r="B160" t="s">
+    </row>
+    <row r="160" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B160" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C160">
@@ -7996,16 +8032,13 @@
       <c r="AD160" s="4"/>
       <c r="AE160" s="4"/>
       <c r="AF160" s="4"/>
-      <c r="AG160" t="s">
-        <v>35</v>
-      </c>
       <c r="AL160">
         <f>AL157/3</f>
         <v>91.706666666666635</v>
       </c>
     </row>
-    <row r="161" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B161" t="s">
+    <row r="161" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B161" s="3" t="s">
         <v>76</v>
       </c>
       <c r="C161">
@@ -8035,12 +8068,9 @@
       <c r="AD161" s="4"/>
       <c r="AE161" s="4"/>
       <c r="AF161" s="4"/>
-      <c r="AG161" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="162" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B162" t="s">
+    </row>
+    <row r="162" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B162" s="3" t="s">
         <v>76</v>
       </c>
       <c r="C162">
@@ -8073,12 +8103,9 @@
       <c r="AD162" s="4"/>
       <c r="AE162" s="4"/>
       <c r="AF162" s="4"/>
-      <c r="AG162" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="163" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B163" t="s">
+    </row>
+    <row r="163" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B163" s="3" t="s">
         <v>85</v>
       </c>
       <c r="C163">
@@ -8112,8 +8139,8 @@
         <v>35</v>
       </c>
     </row>
-    <row r="164" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B164" t="s">
+    <row r="164" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B164" s="3" t="s">
         <v>85</v>
       </c>
       <c r="C164">
@@ -8155,8 +8182,8 @@
         <v>35</v>
       </c>
     </row>
-    <row r="165" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B165" t="s">
+    <row r="165" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B165" s="3" t="s">
         <v>83</v>
       </c>
       <c r="C165">
@@ -8186,9 +8213,12 @@
       <c r="AD165" s="4"/>
       <c r="AE165" s="4"/>
       <c r="AF165" s="4"/>
+      <c r="AG165" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="166" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B166" t="s">
+      <c r="B166" s="3" t="s">
         <v>83</v>
       </c>
       <c r="C166">
@@ -8228,10 +8258,13 @@
       <c r="AD166" s="4"/>
       <c r="AE166" s="4"/>
       <c r="AF166" s="4"/>
-    </row>
-    <row r="167" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B167" t="s">
-        <v>95</v>
+      <c r="AG166" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="167" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B167" s="3" t="s">
+        <v>94</v>
       </c>
       <c r="C167">
         <v>76</v>
@@ -8260,10 +8293,13 @@
       <c r="AD167" s="4"/>
       <c r="AE167" s="4"/>
       <c r="AF167" s="4"/>
+      <c r="AG167" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="168" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B168" t="s">
-        <v>95</v>
+      <c r="B168" s="3" t="s">
+        <v>94</v>
       </c>
       <c r="C168">
         <v>76</v>
@@ -8275,7 +8311,7 @@
         <v>1566.27</v>
       </c>
       <c r="F168" s="3">
-        <v>401</v>
+        <v>531</v>
       </c>
       <c r="L168" s="4"/>
       <c r="M168" s="4"/>
@@ -8295,16 +8331,19 @@
         <v>42</v>
       </c>
       <c r="AA168" s="4">
-        <v>359</v>
+        <v>489</v>
       </c>
       <c r="AB168" s="4"/>
       <c r="AC168" s="4"/>
       <c r="AD168" s="4"/>
       <c r="AE168" s="4"/>
       <c r="AF168" s="4"/>
-    </row>
-    <row r="169" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B169" t="s">
+      <c r="AG168" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="169" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B169" s="3" t="s">
         <v>91</v>
       </c>
       <c r="C169">
@@ -8339,7 +8378,7 @@
       </c>
     </row>
     <row r="170" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B170" t="s">
+      <c r="B170" s="3" t="s">
         <v>91</v>
       </c>
       <c r="C170">
@@ -8385,8 +8424,8 @@
         <v>35</v>
       </c>
     </row>
-    <row r="171" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B171" t="s">
+    <row r="171" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B171" s="3" t="s">
         <v>42</v>
       </c>
       <c r="C171">
@@ -8419,12 +8458,9 @@
       <c r="AD171" s="4"/>
       <c r="AE171" s="4"/>
       <c r="AF171" s="4"/>
-      <c r="AG171" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="172" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B172" t="s">
+    </row>
+    <row r="172" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B172" s="3" t="s">
         <v>42</v>
       </c>
       <c r="C172">
@@ -8454,12 +8490,9 @@
       <c r="AD172" s="4"/>
       <c r="AE172" s="4"/>
       <c r="AF172" s="4"/>
-      <c r="AG172" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="173" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B173" t="s">
+    </row>
+    <row r="173" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B173" s="3" t="s">
         <v>68</v>
       </c>
       <c r="C173">
@@ -8493,8 +8526,8 @@
       <c r="AE173" s="4"/>
       <c r="AF173" s="4"/>
     </row>
-    <row r="174" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B174" t="s">
+    <row r="174" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B174" s="3" t="s">
         <v>68</v>
       </c>
       <c r="C174">
@@ -8528,12 +8561,12 @@
       <c r="AE174" s="4"/>
       <c r="AF174" s="4"/>
     </row>
-    <row r="175" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B175" t="s">
+    <row r="175" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B175" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C175" s="1" t="s">
         <v>98</v>
-      </c>
-      <c r="C175" s="1" t="s">
-        <v>99</v>
       </c>
       <c r="D175" t="s">
         <v>34</v>
@@ -8574,12 +8607,12 @@
       <c r="AE175" s="4"/>
       <c r="AF175" s="4"/>
     </row>
-    <row r="176" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B176" t="s">
+    <row r="176" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B176" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C176" s="1" t="s">
         <v>98</v>
-      </c>
-      <c r="C176" s="1" t="s">
-        <v>99</v>
       </c>
       <c r="D176" t="s">
         <v>36</v>
@@ -8618,12 +8651,12 @@
       <c r="AE176" s="4"/>
       <c r="AF176" s="4"/>
     </row>
-    <row r="177" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B177" t="s">
+    <row r="177" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B177" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C177" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="C177" s="1" t="s">
-        <v>101</v>
       </c>
       <c r="D177" t="s">
         <v>34</v>
@@ -8653,12 +8686,12 @@
       <c r="AE177" s="4"/>
       <c r="AF177" s="4"/>
     </row>
-    <row r="178" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B178" t="s">
+    <row r="178" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B178" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C178" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="C178" s="1" t="s">
-        <v>101</v>
       </c>
       <c r="D178" t="s">
         <v>36</v>
@@ -8688,12 +8721,12 @@
       <c r="AE178" s="4"/>
       <c r="AF178" s="4"/>
     </row>
-    <row r="179" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B179" t="s">
+    <row r="179" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B179" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C179" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="C179" s="1" t="s">
-        <v>103</v>
       </c>
       <c r="D179" t="s">
         <v>34</v>
@@ -8723,12 +8756,12 @@
       <c r="AE179" s="4"/>
       <c r="AF179" s="4"/>
     </row>
-    <row r="180" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B180" t="s">
+    <row r="180" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B180" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C180" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="C180" s="1" t="s">
-        <v>103</v>
       </c>
       <c r="D180" t="s">
         <v>36</v>
@@ -8758,12 +8791,12 @@
       <c r="AE180" s="4"/>
       <c r="AF180" s="4"/>
     </row>
-    <row r="181" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B181" t="s">
+    <row r="181" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B181" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C181" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="C181" s="1" t="s">
-        <v>105</v>
       </c>
       <c r="D181" t="s">
         <v>34</v>
@@ -8789,16 +8822,13 @@
       <c r="AD181" s="4"/>
       <c r="AE181" s="4"/>
       <c r="AF181" s="4"/>
-      <c r="AG181" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="182" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B182" t="s">
+    </row>
+    <row r="182" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B182" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C182" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="C182" s="1" t="s">
-        <v>105</v>
       </c>
       <c r="D182" t="s">
         <v>36</v>
@@ -8827,12 +8857,9 @@
       <c r="AD182" s="4"/>
       <c r="AE182" s="4"/>
       <c r="AF182" s="4"/>
-      <c r="AG182" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="183" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B183" t="s">
+    </row>
+    <row r="183" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B183" s="3" t="s">
         <v>90</v>
       </c>
       <c r="C183">
@@ -8866,8 +8893,8 @@
         <v>40</v>
       </c>
     </row>
-    <row r="184" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B184" t="s">
+    <row r="184" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B184" s="3" t="s">
         <v>90</v>
       </c>
       <c r="C184">
@@ -8900,9 +8927,12 @@
       <c r="AD184" s="4"/>
       <c r="AE184" s="4"/>
       <c r="AF184" s="4"/>
-    </row>
-    <row r="185" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B185" t="s">
+      <c r="AG184" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="185" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B185" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C185">
@@ -8939,8 +8969,8 @@
       <c r="AE185" s="4"/>
       <c r="AF185" s="4"/>
     </row>
-    <row r="186" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B186" t="s">
+    <row r="186" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B186" s="3" t="s">
         <v>78</v>
       </c>
       <c r="C186">
@@ -8974,8 +9004,8 @@
       <c r="AE186" s="4"/>
       <c r="AF186" s="4"/>
     </row>
-    <row r="187" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B187" t="s">
+    <row r="187" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B187" s="3" t="s">
         <v>44</v>
       </c>
       <c r="C187">
@@ -9011,11 +9041,11 @@
       <c r="AE187" s="4"/>
       <c r="AF187" s="4"/>
       <c r="AG187" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="188" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B188" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="188" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B188" s="3" t="s">
         <v>44</v>
       </c>
       <c r="C188">
@@ -9049,11 +9079,11 @@
       <c r="AE188" s="4"/>
       <c r="AF188" s="4"/>
       <c r="AG188" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="189" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B189" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="189" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B189" s="3" t="s">
         <v>45</v>
       </c>
       <c r="C189">
@@ -9084,8 +9114,8 @@
       <c r="AE189" s="4"/>
       <c r="AF189" s="4"/>
     </row>
-    <row r="190" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B190" t="s">
+    <row r="190" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B190" s="3" t="s">
         <v>45</v>
       </c>
       <c r="C190">
@@ -9119,8 +9149,8 @@
       <c r="AE190" s="4"/>
       <c r="AF190" s="4"/>
     </row>
-    <row r="191" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B191" t="s">
+    <row r="191" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B191" s="3" t="s">
         <v>54</v>
       </c>
       <c r="C191">
@@ -9151,8 +9181,8 @@
       <c r="AE191" s="4"/>
       <c r="AF191" s="4"/>
     </row>
-    <row r="192" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B192" t="s">
+    <row r="192" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B192" s="3" t="s">
         <v>54</v>
       </c>
       <c r="C192">
@@ -9187,8 +9217,8 @@
       <c r="AE192" s="4"/>
       <c r="AF192" s="4"/>
     </row>
-    <row r="193" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B193" t="s">
+    <row r="193" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B193" s="3" t="s">
         <v>43</v>
       </c>
       <c r="C193">
@@ -9218,9 +9248,12 @@
       <c r="AD193" s="4"/>
       <c r="AE193" s="4"/>
       <c r="AF193" s="4"/>
-    </row>
-    <row r="194" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B194" t="s">
+      <c r="AG193" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="194" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B194" s="3" t="s">
         <v>43</v>
       </c>
       <c r="C194">
@@ -9253,9 +9286,12 @@
       <c r="AD194" s="4"/>
       <c r="AE194" s="4"/>
       <c r="AF194" s="4"/>
-    </row>
-    <row r="195" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B195" t="s">
+      <c r="AG194" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="195" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B195" s="3" t="s">
         <v>92</v>
       </c>
       <c r="C195">
@@ -9288,12 +9324,9 @@
       <c r="AD195" s="4"/>
       <c r="AE195" s="4"/>
       <c r="AF195" s="4"/>
-      <c r="AG195" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="196" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B196" t="s">
+    </row>
+    <row r="196" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B196" s="3" t="s">
         <v>92</v>
       </c>
       <c r="C196">
@@ -9326,12 +9359,9 @@
       <c r="AD196" s="4"/>
       <c r="AE196" s="4"/>
       <c r="AF196" s="4"/>
-      <c r="AG196" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="197" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B197" t="s">
+    </row>
+    <row r="197" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B197" s="3" t="s">
         <v>46</v>
       </c>
       <c r="C197">
@@ -9361,12 +9391,9 @@
       <c r="AD197" s="4"/>
       <c r="AE197" s="4"/>
       <c r="AF197" s="4"/>
-      <c r="AG197" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="198" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B198" t="s">
+    </row>
+    <row r="198" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B198" s="3" t="s">
         <v>46</v>
       </c>
       <c r="C198">
@@ -9399,12 +9426,9 @@
       <c r="AD198" s="4"/>
       <c r="AE198" s="4"/>
       <c r="AF198" s="4"/>
-      <c r="AG198" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="199" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B199" t="s">
+    </row>
+    <row r="199" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B199" s="3" t="s">
         <v>41</v>
       </c>
       <c r="C199">
@@ -9437,12 +9461,9 @@
       <c r="AD199" s="4"/>
       <c r="AE199" s="4"/>
       <c r="AF199" s="4"/>
-      <c r="AG199" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="200" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B200" t="s">
+    </row>
+    <row r="200" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B200" s="3" t="s">
         <v>41</v>
       </c>
       <c r="C200">
@@ -9475,12 +9496,9 @@
       <c r="AD200" s="4"/>
       <c r="AE200" s="4"/>
       <c r="AF200" s="4"/>
-      <c r="AG200" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="201" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B201" t="s">
+    </row>
+    <row r="201" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B201" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C201">
@@ -9510,12 +9528,9 @@
       <c r="AD201" s="4"/>
       <c r="AE201" s="4"/>
       <c r="AF201" s="4"/>
-      <c r="AG201" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="202" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B202" t="s">
+    </row>
+    <row r="202" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B202" s="3" t="s">
         <v>61</v>
       </c>
       <c r="C202">
@@ -9548,13 +9563,10 @@
       <c r="AD202" s="4"/>
       <c r="AE202" s="4"/>
       <c r="AF202" s="4"/>
-      <c r="AG202" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="203" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B203" t="s">
-        <v>96</v>
+    </row>
+    <row r="203" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B203" s="3" t="s">
+        <v>95</v>
       </c>
       <c r="C203">
         <v>76</v>
@@ -9587,9 +9599,9 @@
         <v>35</v>
       </c>
     </row>
-    <row r="204" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B204" t="s">
-        <v>96</v>
+    <row r="204" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B204" s="3" t="s">
+        <v>95</v>
       </c>
       <c r="C204">
         <v>76</v>
@@ -9630,8 +9642,8 @@
         <v>35</v>
       </c>
     </row>
-    <row r="205" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B205" t="s">
+    <row r="205" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B205" s="3" t="s">
         <v>69</v>
       </c>
       <c r="C205">
@@ -9675,7 +9687,7 @@
       </c>
     </row>
     <row r="206" spans="2:33" x14ac:dyDescent="0.3">
-      <c r="B206" t="s">
+      <c r="B206" s="3" t="s">
         <v>69</v>
       </c>
       <c r="C206">
@@ -9688,7 +9700,7 @@
         <v>1799.2</v>
       </c>
       <c r="F206" s="3">
-        <v>1696.2</v>
+        <v>1716.2</v>
       </c>
       <c r="L206" s="4"/>
       <c r="M206" s="4"/>
@@ -9710,7 +9722,7 @@
         <v>584.20000000000005</v>
       </c>
       <c r="AA206" s="4">
-        <v>182</v>
+        <v>202</v>
       </c>
       <c r="AB206" s="4"/>
       <c r="AC206" s="4"/>
@@ -9721,7 +9733,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="207" spans="2:33" x14ac:dyDescent="0.3">
+    <row r="207" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B207" t="s">
         <v>72</v>
       </c>
@@ -9755,9 +9767,6 @@
       <c r="AD207" s="4"/>
       <c r="AE207" s="4"/>
       <c r="AF207" s="4"/>
-      <c r="AG207" t="s">
-        <v>35</v>
-      </c>
     </row>
     <row r="208" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B208" t="s">
@@ -9773,7 +9782,7 @@
         <v>382.5</v>
       </c>
       <c r="F208" s="3">
-        <v>68</v>
+        <v>126</v>
       </c>
       <c r="L208" s="4"/>
       <c r="M208" s="4"/>
@@ -9791,18 +9800,15 @@
       <c r="Y208" s="4"/>
       <c r="Z208" s="9"/>
       <c r="AA208" s="4">
-        <v>68</v>
+        <v>126</v>
       </c>
       <c r="AB208" s="4"/>
       <c r="AC208" s="4"/>
       <c r="AD208" s="4"/>
       <c r="AE208" s="4"/>
       <c r="AF208" s="4"/>
-      <c r="AG208" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="209" spans="2:33" x14ac:dyDescent="0.3">
+    </row>
+    <row r="209" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B209" t="s">
         <v>84</v>
       </c>
@@ -9839,11 +9845,8 @@
       <c r="AD209" s="4"/>
       <c r="AE209" s="4"/>
       <c r="AF209" s="4"/>
-      <c r="AG209" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="210" spans="2:33" x14ac:dyDescent="0.3">
+    </row>
+    <row r="210" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B210" t="s">
         <v>84</v>
       </c>
@@ -9877,13 +9880,10 @@
       <c r="AD210" s="4"/>
       <c r="AE210" s="4"/>
       <c r="AF210" s="4"/>
-      <c r="AG210" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="211" spans="2:33" x14ac:dyDescent="0.3">
+    </row>
+    <row r="211" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B211" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C211">
         <v>76</v>
@@ -9912,13 +9912,10 @@
       <c r="AD211" s="4"/>
       <c r="AE211" s="4"/>
       <c r="AF211" s="4"/>
-      <c r="AG211" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="212" spans="2:33" x14ac:dyDescent="0.3">
+    </row>
+    <row r="212" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B212" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C212">
         <v>76</v>
@@ -9950,11 +9947,8 @@
       <c r="AD212" s="4"/>
       <c r="AE212" s="4"/>
       <c r="AF212" s="4"/>
-      <c r="AG212" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="213" spans="2:33" x14ac:dyDescent="0.3">
+    </row>
+    <row r="213" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B213" t="s">
         <v>75</v>
       </c>
@@ -9991,11 +9985,8 @@
       <c r="AD213" s="4"/>
       <c r="AE213" s="4"/>
       <c r="AF213" s="4"/>
-      <c r="AG213" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="214" spans="2:33" x14ac:dyDescent="0.3">
+    </row>
+    <row r="214" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B214" t="s">
         <v>75</v>
       </c>
@@ -10029,11 +10020,8 @@
       <c r="AD214" s="4"/>
       <c r="AE214" s="4"/>
       <c r="AF214" s="4"/>
-      <c r="AG214" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="215" spans="2:33" x14ac:dyDescent="0.3">
+    </row>
+    <row r="215" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B215" t="s">
         <v>73</v>
       </c>
@@ -10067,11 +10055,8 @@
       <c r="AD215" s="4"/>
       <c r="AE215" s="4"/>
       <c r="AF215" s="4"/>
-      <c r="AG215" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="216" spans="2:33" x14ac:dyDescent="0.3">
+    </row>
+    <row r="216" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B216" t="s">
         <v>73</v>
       </c>
@@ -10105,11 +10090,8 @@
       <c r="AD216" s="4"/>
       <c r="AE216" s="4"/>
       <c r="AF216" s="4"/>
-      <c r="AG216" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="217" spans="2:33" x14ac:dyDescent="0.3">
+    </row>
+    <row r="217" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B217" t="s">
         <v>39</v>
       </c>
@@ -10147,10 +10129,10 @@
       <c r="AE217" s="4"/>
       <c r="AF217" s="4"/>
       <c r="AG217" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="218" spans="2:33" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="218" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
       <c r="B218" t="s">
         <v>39</v>
       </c>
@@ -10182,15 +10164,15 @@
       <c r="AE218" s="4"/>
       <c r="AF218" s="4"/>
       <c r="AG218" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="AG1:AG218" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -10212,19 +10194,19 @@
   <sheetData>
     <row r="2" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C2" t="s">
         <v>106</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>107</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>108</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>109</v>
-      </c>
-      <c r="F2" t="s">
-        <v>110</v>
       </c>
       <c r="G2" t="s">
         <v>9</v>
@@ -10235,7 +10217,7 @@
         <v>2025</v>
       </c>
       <c r="C3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D3">
         <v>159.15</v>
@@ -10255,7 +10237,7 @@
         <v>2025</v>
       </c>
       <c r="C4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D4">
         <v>723.7</v>
@@ -10275,7 +10257,7 @@
         <v>2025</v>
       </c>
       <c r="C5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D5">
         <v>905.99</v>
@@ -10295,7 +10277,7 @@
         <v>2025</v>
       </c>
       <c r="C6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D6">
         <v>1089.1400000000001</v>
@@ -10319,7 +10301,7 @@
         <v>2025</v>
       </c>
       <c r="C7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D7">
         <v>588.28</v>
@@ -10343,7 +10325,7 @@
         <v>2025</v>
       </c>
       <c r="C8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D8">
         <v>1227.24</v>
@@ -10367,7 +10349,7 @@
         <v>2025</v>
       </c>
       <c r="C9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D9">
         <v>1914.65</v>
@@ -10395,7 +10377,7 @@
         <v>2025</v>
       </c>
       <c r="C10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D10">
         <v>1749.47</v>
@@ -10423,7 +10405,7 @@
         <v>2025</v>
       </c>
       <c r="C11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D11">
         <v>1942.9</v>
@@ -10451,7 +10433,7 @@
         <v>2025</v>
       </c>
       <c r="C12" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D12">
         <v>1588.61</v>
@@ -10475,7 +10457,7 @@
         <v>2026</v>
       </c>
       <c r="C13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D13">
         <v>2185.34</v>
@@ -10499,7 +10481,7 @@
         <v>2026</v>
       </c>
       <c r="C14" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D14">
         <v>2340.4</v>
@@ -10523,7 +10505,7 @@
         <v>2026</v>
       </c>
       <c r="C15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D15">
         <v>2128.08</v>
@@ -10542,7 +10524,7 @@
         <v>539.41999999999985</v>
       </c>
       <c r="O15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="16" spans="2:15" x14ac:dyDescent="0.3">
@@ -10550,7 +10532,7 @@
         <v>2026</v>
       </c>
       <c r="C16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D16">
         <v>2426.84</v>
@@ -10574,7 +10556,7 @@
         <v>2026</v>
       </c>
       <c r="C17" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D17">
         <v>2545.85</v>
@@ -10599,7 +10581,7 @@
         <v>2026</v>
       </c>
       <c r="C18" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D18">
         <v>3108.25</v>
@@ -10616,7 +10598,7 @@
         <v>2026</v>
       </c>
       <c r="C19" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D19">
         <v>3269.49</v>
@@ -10633,7 +10615,7 @@
         <v>2026</v>
       </c>
       <c r="C20" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D20">
         <v>3305.21</v>
@@ -10650,7 +10632,7 @@
         <v>2026</v>
       </c>
       <c r="C21" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D21">
         <v>3138.09</v>
@@ -10667,7 +10649,7 @@
         <v>2026</v>
       </c>
       <c r="C22" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D22">
         <v>2251.2800000000002</v>
@@ -10684,7 +10666,7 @@
         <v>2026</v>
       </c>
       <c r="C23" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D23">
         <v>1527.07</v>
@@ -10701,7 +10683,7 @@
         <v>2026</v>
       </c>
       <c r="C24" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D24">
         <v>542.46</v>
@@ -10733,7 +10715,7 @@
     </row>
     <row r="34" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H34" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza dashboard em 2026-07-22
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A6D93DF-D2A3-4536-BFA7-4CF39D87C8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16FE1838-5364-4E8C-B508-E8192FBD5A01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BASE_DASH_EXTENSAO" sheetId="1" r:id="rId1"/>
@@ -796,13 +796,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tb_base_dash_extensao" displayName="tb_base_dash_extensao" ref="B1:AF218">
-  <autoFilter ref="B1:AF218" xr:uid="{00000000-0009-0000-0100-000001000000}">
-    <filterColumn colId="25">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="B1:AF218" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:AF218">
     <sortCondition ref="B1:B218"/>
   </sortState>
@@ -1256,7 +1250,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B2" s="3" t="s">
         <v>64</v>
       </c>
@@ -1313,7 +1307,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B3" s="3" t="s">
         <v>64</v>
       </c>
@@ -1356,7 +1350,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>64</v>
       </c>
@@ -1402,7 +1396,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B5" s="3" t="s">
         <v>64</v>
       </c>
@@ -1445,7 +1439,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
         <v>64</v>
       </c>
@@ -1491,7 +1485,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B7" s="3" t="s">
         <v>64</v>
       </c>
@@ -1534,7 +1528,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B8" s="3" t="s">
         <v>63</v>
       </c>
@@ -1582,7 +1576,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B9" s="3" t="s">
         <v>63</v>
       </c>
@@ -1625,7 +1619,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B10" s="3" t="s">
         <v>63</v>
       </c>
@@ -1670,7 +1664,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B11" s="3" t="s">
         <v>63</v>
       </c>
@@ -1708,7 +1702,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B12" s="3" t="s">
         <v>63</v>
       </c>
@@ -1751,7 +1745,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B13" s="3" t="s">
         <v>63</v>
       </c>
@@ -1789,7 +1783,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
         <v>63</v>
       </c>
@@ -1834,7 +1828,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B15" s="3" t="s">
         <v>63</v>
       </c>
@@ -1872,7 +1866,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
         <v>63</v>
       </c>
@@ -1917,7 +1911,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B17" s="3" t="s">
         <v>63</v>
       </c>
@@ -1955,7 +1949,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="18" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B18" s="3" t="s">
         <v>63</v>
       </c>
@@ -1998,7 +1992,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B19" s="3" t="s">
         <v>63</v>
       </c>
@@ -2036,7 +2030,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B20" s="3" t="s">
         <v>63</v>
       </c>
@@ -2079,7 +2073,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="21" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B21" s="3" t="s">
         <v>63</v>
       </c>
@@ -2117,7 +2111,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B22" s="3" t="s">
         <v>63</v>
       </c>
@@ -2160,7 +2154,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B23" s="3" t="s">
         <v>63</v>
       </c>
@@ -2198,7 +2192,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="24" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B24" s="3" t="s">
         <v>63</v>
       </c>
@@ -2243,7 +2237,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="25" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B25" s="3" t="s">
         <v>63</v>
       </c>
@@ -2284,7 +2278,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B26" s="3" t="s">
         <v>62</v>
       </c>
@@ -2329,7 +2323,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="27" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B27" s="3" t="s">
         <v>62</v>
       </c>
@@ -2374,7 +2368,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="28" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B28" s="3" t="s">
         <v>62</v>
       </c>
@@ -2417,7 +2411,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="29" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
         <v>62</v>
       </c>
@@ -2455,7 +2449,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="30" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B30" s="3" t="s">
         <v>62</v>
       </c>
@@ -2495,7 +2489,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B31" s="3" t="s">
         <v>62</v>
       </c>
@@ -2533,7 +2527,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="32" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B32" s="3" t="s">
         <v>62</v>
       </c>
@@ -2573,7 +2567,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="33" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B33" s="3" t="s">
         <v>62</v>
       </c>
@@ -2611,7 +2605,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="34" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B34" s="3" t="s">
         <v>62</v>
       </c>
@@ -2654,7 +2648,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="35" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B35" s="3" t="s">
         <v>62</v>
       </c>
@@ -2692,7 +2686,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="36" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B36" s="3" t="s">
         <v>62</v>
       </c>
@@ -2732,7 +2726,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B37" s="3" t="s">
         <v>62</v>
       </c>
@@ -2770,7 +2764,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="38" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B38" s="3" t="s">
         <v>62</v>
       </c>
@@ -2810,7 +2804,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="39" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B39" s="3" t="s">
         <v>62</v>
       </c>
@@ -2848,7 +2842,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="40" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B40" s="3" t="s">
         <v>62</v>
       </c>
@@ -2888,7 +2882,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="41" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B41" s="3" t="s">
         <v>62</v>
       </c>
@@ -2926,7 +2920,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="42" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B42" s="3" t="s">
         <v>62</v>
       </c>
@@ -2966,7 +2960,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="43" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B43" s="3" t="s">
         <v>62</v>
       </c>
@@ -3004,7 +2998,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="44" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B44" s="3" t="s">
         <v>62</v>
       </c>
@@ -3047,7 +3041,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="45" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B45" s="3" t="s">
         <v>62</v>
       </c>
@@ -3085,7 +3079,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="46" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B46" s="3" t="s">
         <v>62</v>
       </c>
@@ -3130,7 +3124,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="47" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B47" s="3" t="s">
         <v>62</v>
       </c>
@@ -3168,7 +3162,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="48" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B48" s="3" t="s">
         <v>62</v>
       </c>
@@ -3213,7 +3207,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="49" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B49" s="3" t="s">
         <v>62</v>
       </c>
@@ -3251,7 +3245,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="50" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B50" s="3" t="s">
         <v>62</v>
       </c>
@@ -3294,7 +3288,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="51" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B51" s="3" t="s">
         <v>62</v>
       </c>
@@ -3332,7 +3326,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="52" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B52" s="3" t="s">
         <v>62</v>
       </c>
@@ -3375,7 +3369,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="53" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B53" s="3" t="s">
         <v>62</v>
       </c>
@@ -3413,7 +3407,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="54" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B54" s="3" t="s">
         <v>62</v>
       </c>
@@ -3458,7 +3452,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="55" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B55" s="3" t="s">
         <v>62</v>
       </c>
@@ -3496,7 +3490,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="56" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B56" s="3" t="s">
         <v>62</v>
       </c>
@@ -3542,7 +3536,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="57" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B57" s="3" t="s">
         <v>62</v>
       </c>
@@ -3585,7 +3579,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="58" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B58" s="3" t="s">
         <v>62</v>
       </c>
@@ -3628,7 +3622,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="59" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B59" s="3" t="s">
         <v>62</v>
       </c>
@@ -3666,7 +3660,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="60" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B60" s="3" t="s">
         <v>58</v>
       </c>
@@ -3731,7 +3725,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="61" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B61" s="3" t="s">
         <v>58</v>
       </c>
@@ -3774,7 +3768,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="62" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B62" s="3" t="s">
         <v>58</v>
       </c>
@@ -3830,7 +3824,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="63" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B63" s="3" t="s">
         <v>58</v>
       </c>
@@ -3872,7 +3866,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="64" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B64" s="3" t="s">
         <v>58</v>
       </c>
@@ -3930,7 +3924,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="65" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B65" s="3" t="s">
         <v>58</v>
       </c>
@@ -3974,7 +3968,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="66" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B66" s="3" t="s">
         <v>59</v>
       </c>
@@ -4021,7 +4015,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="67" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B67" s="3" t="s">
         <v>59</v>
       </c>
@@ -4066,7 +4060,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="68" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B68" s="3" t="s">
         <v>59</v>
       </c>
@@ -4113,7 +4107,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="69" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B69" s="3" t="s">
         <v>59</v>
       </c>
@@ -4157,7 +4151,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="70" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B70" s="3" t="s">
         <v>33</v>
       </c>
@@ -4203,7 +4197,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="71" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B71" s="3" t="s">
         <v>33</v>
       </c>
@@ -4246,7 +4240,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="72" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B72" s="3" t="s">
         <v>33</v>
       </c>
@@ -4291,7 +4285,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="73" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B73" s="3" t="s">
         <v>33</v>
       </c>
@@ -4334,7 +4328,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="74" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B74" s="3" t="s">
         <v>33</v>
       </c>
@@ -4377,7 +4371,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="75" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B75" s="3" t="s">
         <v>33</v>
       </c>
@@ -4420,7 +4414,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="76" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B76" s="3" t="s">
         <v>33</v>
       </c>
@@ -4468,7 +4462,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="77" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B77" s="3" t="s">
         <v>33</v>
       </c>
@@ -4512,7 +4506,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="78" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B78" s="3" t="s">
         <v>38</v>
       </c>
@@ -4567,7 +4561,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="79" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B79" s="3" t="s">
         <v>38</v>
       </c>
@@ -4610,7 +4604,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="80" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B80" s="3" t="s">
         <v>38</v>
       </c>
@@ -4659,7 +4653,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="81" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B81" s="3" t="s">
         <v>38</v>
       </c>
@@ -4702,7 +4696,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="82" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B82" s="3" t="s">
         <v>60</v>
       </c>
@@ -4751,7 +4745,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="83" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B83" s="3" t="s">
         <v>60</v>
       </c>
@@ -4794,7 +4788,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="84" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B84" s="3" t="s">
         <v>57</v>
       </c>
@@ -4850,7 +4844,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="85" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B85" s="3" t="s">
         <v>57</v>
       </c>
@@ -4894,7 +4888,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="86" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B86" s="3" t="s">
         <v>57</v>
       </c>
@@ -4944,7 +4938,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="87" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B87" s="3" t="s">
         <v>57</v>
       </c>
@@ -4988,7 +4982,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="88" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B88" s="3" t="s">
         <v>57</v>
       </c>
@@ -5040,7 +5034,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="89" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B89" s="3" t="s">
         <v>57</v>
       </c>
@@ -5084,7 +5078,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="90" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B90" t="s">
         <v>52</v>
       </c>
@@ -5119,7 +5113,7 @@
       <c r="AE90" s="4"/>
       <c r="AF90" s="4"/>
     </row>
-    <row r="91" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B91" t="s">
         <v>52</v>
       </c>
@@ -5154,7 +5148,7 @@
       <c r="AE91" s="4"/>
       <c r="AF91" s="4"/>
     </row>
-    <row r="92" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B92" s="3" t="s">
         <v>56</v>
       </c>
@@ -5206,7 +5200,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="93" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B93" s="3" t="s">
         <v>56</v>
       </c>
@@ -5248,7 +5242,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="94" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B94" s="3" t="s">
         <v>56</v>
       </c>
@@ -5300,7 +5294,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="95" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B95" s="3" t="s">
         <v>56</v>
       </c>
@@ -5342,7 +5336,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="96" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B96" s="3" t="s">
         <v>56</v>
       </c>
@@ -5394,7 +5388,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="97" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B97" s="3" t="s">
         <v>56</v>
       </c>
@@ -5438,7 +5432,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="98" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B98" s="3" t="s">
         <v>56</v>
       </c>
@@ -5485,7 +5479,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="99" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B99" s="3" t="s">
         <v>56</v>
       </c>
@@ -5529,7 +5523,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="100" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B100" s="3" t="s">
         <v>55</v>
       </c>
@@ -5576,7 +5570,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="101" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B101" s="3" t="s">
         <v>37</v>
       </c>
@@ -5633,7 +5627,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="102" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B102" s="3" t="s">
         <v>37</v>
       </c>
@@ -5671,7 +5665,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="103" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B103" s="3" t="s">
         <v>37</v>
       </c>
@@ -5722,7 +5716,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="104" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B104" s="3" t="s">
         <v>37</v>
       </c>
@@ -5763,7 +5757,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="105" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B105" s="3" t="s">
         <v>37</v>
       </c>
@@ -5814,7 +5808,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="106" spans="2:33" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B106" s="3" t="s">
         <v>37</v>
       </c>
@@ -5857,7 +5851,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="107" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B107" s="3" t="s">
         <v>37</v>
       </c>
@@ -5910,7 +5904,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="108" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B108" s="3" t="s">
         <v>37</v>
       </c>
@@ -5948,7 +5942,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="109" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B109" s="3" t="s">
         <v>37</v>
       </c>
@@ -5997,7 +5991,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="110" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B110" s="3" t="s">
         <v>37</v>
       </c>
@@ -6046,7 +6040,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="111" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B111" t="s">
         <v>89</v>
       </c>
@@ -6090,7 +6084,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="112" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B112" t="s">
         <v>89</v>
       </c>
@@ -6128,7 +6122,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="113" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B113" s="3" t="s">
         <v>77</v>
       </c>
@@ -6174,7 +6168,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="114" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B114" s="3" t="s">
         <v>77</v>
       </c>
@@ -6212,7 +6206,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="115" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B115" s="3" t="s">
         <v>77</v>
       </c>
@@ -6261,7 +6255,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="116" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B116" s="3" t="s">
         <v>77</v>
       </c>
@@ -6304,7 +6298,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="117" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B117" s="3" t="s">
         <v>74</v>
       </c>
@@ -6365,7 +6359,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="118" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B118" s="3" t="s">
         <v>74</v>
       </c>
@@ -6414,7 +6408,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="119" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B119" s="3" t="s">
         <v>74</v>
       </c>
@@ -6473,7 +6467,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="120" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B120" s="3" t="s">
         <v>74</v>
       </c>
@@ -6519,7 +6513,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="121" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B121" s="3" t="s">
         <v>74</v>
       </c>
@@ -6568,7 +6562,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="122" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B122" s="3" t="s">
         <v>74</v>
       </c>
@@ -6611,7 +6605,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="123" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B123" t="s">
         <v>50</v>
       </c>
@@ -6646,7 +6640,7 @@
       <c r="AE123" s="4"/>
       <c r="AF123" s="4"/>
     </row>
-    <row r="124" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B124" t="s">
         <v>50</v>
       </c>
@@ -6678,7 +6672,7 @@
       <c r="AE124" s="4"/>
       <c r="AF124" s="4"/>
     </row>
-    <row r="125" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B125" t="s">
         <v>53</v>
       </c>
@@ -6713,7 +6707,7 @@
       <c r="AE125" s="4"/>
       <c r="AF125" s="4"/>
     </row>
-    <row r="126" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B126" t="s">
         <v>53</v>
       </c>
@@ -6748,7 +6742,7 @@
       <c r="AE126" s="4"/>
       <c r="AF126" s="4"/>
     </row>
-    <row r="127" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B127" t="s">
         <v>48</v>
       </c>
@@ -6783,7 +6777,7 @@
       <c r="AE127" s="4"/>
       <c r="AF127" s="4"/>
     </row>
-    <row r="128" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B128" t="s">
         <v>48</v>
       </c>
@@ -6815,7 +6809,7 @@
       <c r="AE128" s="4"/>
       <c r="AF128" s="4"/>
     </row>
-    <row r="129" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B129" t="s">
         <v>70</v>
       </c>
@@ -6847,7 +6841,7 @@
       <c r="AE129" s="4"/>
       <c r="AF129" s="4"/>
     </row>
-    <row r="130" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B130" t="s">
         <v>70</v>
       </c>
@@ -6882,7 +6876,7 @@
       <c r="AE130" s="4"/>
       <c r="AF130" s="4"/>
     </row>
-    <row r="131" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B131" s="3" t="s">
         <v>82</v>
       </c>
@@ -6931,7 +6925,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="132" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B132" s="3" t="s">
         <v>82</v>
       </c>
@@ -6975,7 +6969,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="133" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B133" s="3" t="s">
         <v>71</v>
       </c>
@@ -7013,7 +7007,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="134" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B134" s="3" t="s">
         <v>71</v>
       </c>
@@ -7056,7 +7050,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="135" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B135" s="3" t="s">
         <v>80</v>
       </c>
@@ -7097,7 +7091,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="136" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B136" s="3" t="s">
         <v>80</v>
       </c>
@@ -7135,7 +7129,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="137" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B137" s="3" t="s">
         <v>51</v>
       </c>
@@ -7170,7 +7164,7 @@
       <c r="AE137" s="4"/>
       <c r="AF137" s="4"/>
     </row>
-    <row r="138" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B138" s="3" t="s">
         <v>51</v>
       </c>
@@ -7205,7 +7199,7 @@
       <c r="AE138" s="4"/>
       <c r="AF138" s="4"/>
     </row>
-    <row r="139" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B139" s="3" t="s">
         <v>49</v>
       </c>
@@ -7240,7 +7234,7 @@
       <c r="AE139" s="4"/>
       <c r="AF139" s="4"/>
     </row>
-    <row r="140" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B140" s="3" t="s">
         <v>49</v>
       </c>
@@ -7272,7 +7266,7 @@
       <c r="AE140" s="4"/>
       <c r="AF140" s="4"/>
     </row>
-    <row r="141" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B141" s="3" t="s">
         <v>81</v>
       </c>
@@ -7304,7 +7298,7 @@
       <c r="AE141" s="4"/>
       <c r="AF141" s="4"/>
     </row>
-    <row r="142" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B142" s="3" t="s">
         <v>81</v>
       </c>
@@ -7339,7 +7333,7 @@
       <c r="AE142" s="4"/>
       <c r="AF142" s="4"/>
     </row>
-    <row r="143" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B143" s="3" t="s">
         <v>47</v>
       </c>
@@ -7388,7 +7382,7 @@
         <v>205</v>
       </c>
       <c r="F144" s="3">
-        <v>216.1</v>
+        <v>211.95</v>
       </c>
       <c r="L144" s="4"/>
       <c r="M144" s="4"/>
@@ -7408,7 +7402,8 @@
         <v>169.1</v>
       </c>
       <c r="AA144" s="4">
-        <v>47</v>
+        <f>47-4.15</f>
+        <v>42.85</v>
       </c>
       <c r="AB144" s="4"/>
       <c r="AC144" s="4"/>
@@ -7419,7 +7414,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="145" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B145" s="3" t="s">
         <v>65</v>
       </c>
@@ -7468,7 +7463,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="146" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B146" s="3" t="s">
         <v>65</v>
       </c>
@@ -7509,7 +7504,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="147" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B147" s="3" t="s">
         <v>65</v>
       </c>
@@ -7559,7 +7554,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="148" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B148" s="3" t="s">
         <v>65</v>
       </c>
@@ -7604,7 +7599,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="149" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B149" s="3" t="s">
         <v>79</v>
       </c>
@@ -7636,7 +7631,7 @@
       <c r="AE149" s="4"/>
       <c r="AF149" s="4"/>
     </row>
-    <row r="150" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B150" s="3" t="s">
         <v>79</v>
       </c>
@@ -7671,7 +7666,7 @@
       <c r="AE150" s="4"/>
       <c r="AF150" s="4"/>
     </row>
-    <row r="151" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B151" s="3" t="s">
         <v>66</v>
       </c>
@@ -7714,7 +7709,7 @@
       <c r="AE151" s="4"/>
       <c r="AF151" s="4"/>
     </row>
-    <row r="152" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B152" s="3" t="s">
         <v>66</v>
       </c>
@@ -7749,7 +7744,7 @@
       <c r="AE152" s="4"/>
       <c r="AF152" s="4"/>
     </row>
-    <row r="153" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B153" s="3" t="s">
         <v>67</v>
       </c>
@@ -7787,7 +7782,7 @@
       <c r="AE153" s="4"/>
       <c r="AF153" s="4"/>
     </row>
-    <row r="154" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B154" s="3" t="s">
         <v>67</v>
       </c>
@@ -7822,7 +7817,7 @@
       <c r="AE154" s="4"/>
       <c r="AF154" s="4"/>
     </row>
-    <row r="155" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B155" s="3" t="s">
         <v>86</v>
       </c>
@@ -7857,7 +7852,7 @@
         <v>1746.61</v>
       </c>
     </row>
-    <row r="156" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B156" s="3" t="s">
         <v>86</v>
       </c>
@@ -7895,7 +7890,7 @@
         <v>1471.49</v>
       </c>
     </row>
-    <row r="157" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B157" s="3" t="s">
         <v>87</v>
       </c>
@@ -7931,7 +7926,7 @@
         <v>275.11999999999989</v>
       </c>
     </row>
-    <row r="158" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B158" s="3" t="s">
         <v>87</v>
       </c>
@@ -7966,7 +7961,7 @@
       <c r="AE158" s="4"/>
       <c r="AF158" s="4"/>
     </row>
-    <row r="159" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B159" s="3" t="s">
         <v>88</v>
       </c>
@@ -7998,7 +7993,7 @@
       <c r="AE159" s="4"/>
       <c r="AF159" s="4"/>
     </row>
-    <row r="160" spans="2:38" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="2:38" x14ac:dyDescent="0.3">
       <c r="B160" s="3" t="s">
         <v>88</v>
       </c>
@@ -8037,7 +8032,7 @@
         <v>91.706666666666635</v>
       </c>
     </row>
-    <row r="161" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B161" s="3" t="s">
         <v>76</v>
       </c>
@@ -8069,7 +8064,7 @@
       <c r="AE161" s="4"/>
       <c r="AF161" s="4"/>
     </row>
-    <row r="162" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B162" s="3" t="s">
         <v>76</v>
       </c>
@@ -8104,7 +8099,7 @@
       <c r="AE162" s="4"/>
       <c r="AF162" s="4"/>
     </row>
-    <row r="163" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B163" s="3" t="s">
         <v>85</v>
       </c>
@@ -8139,7 +8134,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="164" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B164" s="3" t="s">
         <v>85</v>
       </c>
@@ -8153,7 +8148,7 @@
         <v>338.5</v>
       </c>
       <c r="F164" s="3">
-        <v>377.8</v>
+        <v>390.49</v>
       </c>
       <c r="L164" s="4"/>
       <c r="M164" s="4"/>
@@ -8182,7 +8177,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="165" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B165" s="3" t="s">
         <v>83</v>
       </c>
@@ -8251,7 +8246,8 @@
         <v>100.7</v>
       </c>
       <c r="AA166" s="4">
-        <v>110</v>
+        <f>12.69+110</f>
+        <v>122.69</v>
       </c>
       <c r="AB166" s="4"/>
       <c r="AC166" s="4"/>
@@ -8262,7 +8258,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="167" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B167" s="3" t="s">
         <v>94</v>
       </c>
@@ -8311,7 +8307,7 @@
         <v>1566.27</v>
       </c>
       <c r="F168" s="3">
-        <v>531</v>
+        <v>561</v>
       </c>
       <c r="L168" s="4"/>
       <c r="M168" s="4"/>
@@ -8331,7 +8327,7 @@
         <v>42</v>
       </c>
       <c r="AA168" s="4">
-        <v>489</v>
+        <v>519</v>
       </c>
       <c r="AB168" s="4"/>
       <c r="AC168" s="4"/>
@@ -8342,7 +8338,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="169" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B169" s="3" t="s">
         <v>91</v>
       </c>
@@ -8391,7 +8387,7 @@
         <v>180</v>
       </c>
       <c r="F170" s="3">
-        <v>167.96</v>
+        <v>201.41</v>
       </c>
       <c r="L170" s="4"/>
       <c r="M170" s="4"/>
@@ -8407,7 +8403,8 @@
       <c r="W170" s="4"/>
       <c r="X170" s="4"/>
       <c r="Y170" s="4">
-        <v>43.66</v>
+        <f>33.45+43.66</f>
+        <v>77.11</v>
       </c>
       <c r="Z170" s="9">
         <v>89.8</v>
@@ -8424,7 +8421,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="171" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B171" s="3" t="s">
         <v>42</v>
       </c>
@@ -8459,7 +8456,7 @@
       <c r="AE171" s="4"/>
       <c r="AF171" s="4"/>
     </row>
-    <row r="172" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B172" s="3" t="s">
         <v>42</v>
       </c>
@@ -8491,7 +8488,7 @@
       <c r="AE172" s="4"/>
       <c r="AF172" s="4"/>
     </row>
-    <row r="173" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B173" s="3" t="s">
         <v>68</v>
       </c>
@@ -8526,7 +8523,7 @@
       <c r="AE173" s="4"/>
       <c r="AF173" s="4"/>
     </row>
-    <row r="174" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B174" s="3" t="s">
         <v>68</v>
       </c>
@@ -8561,7 +8558,7 @@
       <c r="AE174" s="4"/>
       <c r="AF174" s="4"/>
     </row>
-    <row r="175" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B175" s="3" t="s">
         <v>97</v>
       </c>
@@ -8607,7 +8604,7 @@
       <c r="AE175" s="4"/>
       <c r="AF175" s="4"/>
     </row>
-    <row r="176" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B176" s="3" t="s">
         <v>97</v>
       </c>
@@ -8651,7 +8648,7 @@
       <c r="AE176" s="4"/>
       <c r="AF176" s="4"/>
     </row>
-    <row r="177" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B177" s="3" t="s">
         <v>99</v>
       </c>
@@ -8686,7 +8683,7 @@
       <c r="AE177" s="4"/>
       <c r="AF177" s="4"/>
     </row>
-    <row r="178" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B178" s="3" t="s">
         <v>99</v>
       </c>
@@ -8721,7 +8718,7 @@
       <c r="AE178" s="4"/>
       <c r="AF178" s="4"/>
     </row>
-    <row r="179" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B179" s="3" t="s">
         <v>101</v>
       </c>
@@ -8756,7 +8753,7 @@
       <c r="AE179" s="4"/>
       <c r="AF179" s="4"/>
     </row>
-    <row r="180" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B180" s="3" t="s">
         <v>101</v>
       </c>
@@ -8791,7 +8788,7 @@
       <c r="AE180" s="4"/>
       <c r="AF180" s="4"/>
     </row>
-    <row r="181" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B181" s="3" t="s">
         <v>103</v>
       </c>
@@ -8823,7 +8820,7 @@
       <c r="AE181" s="4"/>
       <c r="AF181" s="4"/>
     </row>
-    <row r="182" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B182" s="3" t="s">
         <v>103</v>
       </c>
@@ -8858,7 +8855,7 @@
       <c r="AE182" s="4"/>
       <c r="AF182" s="4"/>
     </row>
-    <row r="183" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B183" s="3" t="s">
         <v>90</v>
       </c>
@@ -8893,7 +8890,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="184" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B184" s="3" t="s">
         <v>90</v>
       </c>
@@ -8931,7 +8928,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="185" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B185" s="3" t="s">
         <v>78</v>
       </c>
@@ -8969,7 +8966,7 @@
       <c r="AE185" s="4"/>
       <c r="AF185" s="4"/>
     </row>
-    <row r="186" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B186" s="3" t="s">
         <v>78</v>
       </c>
@@ -9004,7 +9001,7 @@
       <c r="AE186" s="4"/>
       <c r="AF186" s="4"/>
     </row>
-    <row r="187" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B187" s="3" t="s">
         <v>44</v>
       </c>
@@ -9044,7 +9041,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="188" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B188" s="3" t="s">
         <v>44</v>
       </c>
@@ -9082,7 +9079,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="189" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B189" s="3" t="s">
         <v>45</v>
       </c>
@@ -9114,7 +9111,7 @@
       <c r="AE189" s="4"/>
       <c r="AF189" s="4"/>
     </row>
-    <row r="190" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B190" s="3" t="s">
         <v>45</v>
       </c>
@@ -9149,7 +9146,7 @@
       <c r="AE190" s="4"/>
       <c r="AF190" s="4"/>
     </row>
-    <row r="191" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B191" s="3" t="s">
         <v>54</v>
       </c>
@@ -9181,7 +9178,7 @@
       <c r="AE191" s="4"/>
       <c r="AF191" s="4"/>
     </row>
-    <row r="192" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B192" s="3" t="s">
         <v>54</v>
       </c>
@@ -9217,7 +9214,7 @@
       <c r="AE192" s="4"/>
       <c r="AF192" s="4"/>
     </row>
-    <row r="193" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B193" s="3" t="s">
         <v>43</v>
       </c>
@@ -9252,7 +9249,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="194" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B194" s="3" t="s">
         <v>43</v>
       </c>
@@ -9290,7 +9287,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="195" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B195" s="3" t="s">
         <v>92</v>
       </c>
@@ -9325,7 +9322,7 @@
       <c r="AE195" s="4"/>
       <c r="AF195" s="4"/>
     </row>
-    <row r="196" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B196" s="3" t="s">
         <v>92</v>
       </c>
@@ -9360,7 +9357,7 @@
       <c r="AE196" s="4"/>
       <c r="AF196" s="4"/>
     </row>
-    <row r="197" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B197" s="3" t="s">
         <v>46</v>
       </c>
@@ -9392,7 +9389,7 @@
       <c r="AE197" s="4"/>
       <c r="AF197" s="4"/>
     </row>
-    <row r="198" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B198" s="3" t="s">
         <v>46</v>
       </c>
@@ -9427,7 +9424,7 @@
       <c r="AE198" s="4"/>
       <c r="AF198" s="4"/>
     </row>
-    <row r="199" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B199" s="3" t="s">
         <v>41</v>
       </c>
@@ -9462,7 +9459,7 @@
       <c r="AE199" s="4"/>
       <c r="AF199" s="4"/>
     </row>
-    <row r="200" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B200" s="3" t="s">
         <v>41</v>
       </c>
@@ -9497,7 +9494,7 @@
       <c r="AE200" s="4"/>
       <c r="AF200" s="4"/>
     </row>
-    <row r="201" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B201" s="3" t="s">
         <v>61</v>
       </c>
@@ -9529,7 +9526,7 @@
       <c r="AE201" s="4"/>
       <c r="AF201" s="4"/>
     </row>
-    <row r="202" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B202" s="3" t="s">
         <v>61</v>
       </c>
@@ -9564,7 +9561,7 @@
       <c r="AE202" s="4"/>
       <c r="AF202" s="4"/>
     </row>
-    <row r="203" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B203" s="3" t="s">
         <v>95</v>
       </c>
@@ -9599,7 +9596,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="204" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B204" s="3" t="s">
         <v>95</v>
       </c>
@@ -9613,7 +9610,7 @@
         <v>95</v>
       </c>
       <c r="F204" s="3">
-        <v>93.2</v>
+        <v>82.99</v>
       </c>
       <c r="L204" s="4"/>
       <c r="M204" s="4"/>
@@ -9629,7 +9626,7 @@
       <c r="W204" s="4"/>
       <c r="X204" s="4"/>
       <c r="Y204" s="4">
-        <v>93.2</v>
+        <v>82.99</v>
       </c>
       <c r="Z204" s="9"/>
       <c r="AA204" s="4"/>
@@ -9642,7 +9639,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="205" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B205" s="3" t="s">
         <v>69</v>
       </c>
@@ -9700,7 +9697,7 @@
         <v>1799.2</v>
       </c>
       <c r="F206" s="3">
-        <v>1716.2</v>
+        <v>1616.26</v>
       </c>
       <c r="L206" s="4"/>
       <c r="M206" s="4"/>
@@ -9716,7 +9713,7 @@
       <c r="W206" s="4"/>
       <c r="X206" s="4"/>
       <c r="Y206" s="4">
-        <v>930</v>
+        <v>830.06</v>
       </c>
       <c r="Z206" s="9">
         <v>584.20000000000005</v>
@@ -9733,7 +9730,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="207" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B207" t="s">
         <v>72</v>
       </c>
@@ -9808,7 +9805,7 @@
       <c r="AE208" s="4"/>
       <c r="AF208" s="4"/>
     </row>
-    <row r="209" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B209" t="s">
         <v>84</v>
       </c>
@@ -9846,7 +9843,7 @@
       <c r="AE209" s="4"/>
       <c r="AF209" s="4"/>
     </row>
-    <row r="210" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B210" t="s">
         <v>84</v>
       </c>
@@ -9881,7 +9878,7 @@
       <c r="AE210" s="4"/>
       <c r="AF210" s="4"/>
     </row>
-    <row r="211" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B211" t="s">
         <v>93</v>
       </c>
@@ -9913,7 +9910,7 @@
       <c r="AE211" s="4"/>
       <c r="AF211" s="4"/>
     </row>
-    <row r="212" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B212" t="s">
         <v>93</v>
       </c>
@@ -9948,7 +9945,7 @@
       <c r="AE212" s="4"/>
       <c r="AF212" s="4"/>
     </row>
-    <row r="213" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B213" t="s">
         <v>75</v>
       </c>
@@ -9986,7 +9983,7 @@
       <c r="AE213" s="4"/>
       <c r="AF213" s="4"/>
     </row>
-    <row r="214" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B214" t="s">
         <v>75</v>
       </c>
@@ -10021,7 +10018,7 @@
       <c r="AE214" s="4"/>
       <c r="AF214" s="4"/>
     </row>
-    <row r="215" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B215" t="s">
         <v>73</v>
       </c>
@@ -10056,7 +10053,7 @@
       <c r="AE215" s="4"/>
       <c r="AF215" s="4"/>
     </row>
-    <row r="216" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B216" t="s">
         <v>73</v>
       </c>
@@ -10091,7 +10088,7 @@
       <c r="AE216" s="4"/>
       <c r="AF216" s="4"/>
     </row>
-    <row r="217" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B217" t="s">
         <v>39</v>
       </c>
@@ -10132,7 +10129,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="218" spans="2:33" hidden="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B218" t="s">
         <v>39</v>
       </c>

</xml_diff>

<commit_message>
Atualiza base de extensao
</commit_message>
<xml_diff>
--- a/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16FE1838-5364-4E8C-B508-E8192FBD5A01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8164927-9F47-4A8C-B1AD-701454278295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4121,7 +4121,7 @@
         <v>194.5</v>
       </c>
       <c r="F69" s="3">
-        <v>12.02</v>
+        <v>13.14</v>
       </c>
       <c r="K69" s="2"/>
       <c r="L69" s="4"/>
@@ -4136,7 +4136,8 @@
       <c r="U69" s="4"/>
       <c r="V69" s="4"/>
       <c r="W69" s="4">
-        <v>12.02</v>
+        <f>12.02+1.12</f>
+        <v>13.14</v>
       </c>
       <c r="X69" s="4"/>
       <c r="Y69" s="4"/>
@@ -6051,7 +6052,7 @@
         <v>34</v>
       </c>
       <c r="F111" s="3">
-        <v>880.94100000000003</v>
+        <v>879.94100000000003</v>
       </c>
       <c r="L111" s="4"/>
       <c r="M111" s="4"/>
@@ -6071,8 +6072,8 @@
         <v>548.55000000000007</v>
       </c>
       <c r="Z111" s="9">
-        <f>64.57+79.57+66.725+63.68+57.846</f>
-        <v>332.39099999999996</v>
+        <f>64.57+79.57+66.725+63.68+56.846</f>
+        <v>331.39099999999996</v>
       </c>
       <c r="AA111" s="4"/>
       <c r="AB111" s="4"/>
@@ -6939,7 +6940,7 @@
         <v>83.8</v>
       </c>
       <c r="F132" s="3">
-        <v>55.83</v>
+        <v>56.52</v>
       </c>
       <c r="L132" s="4"/>
       <c r="M132" s="4"/>
@@ -6954,8 +6955,8 @@
       <c r="V132" s="4"/>
       <c r="W132" s="4"/>
       <c r="X132" s="4">
-        <f>34.75+6.11+14.97</f>
-        <v>55.83</v>
+        <f>34.75+6.11+14.97+0.69</f>
+        <v>56.519999999999996</v>
       </c>
       <c r="Y132" s="4"/>
       <c r="Z132" s="9"/>
@@ -7021,7 +7022,7 @@
         <v>59.5</v>
       </c>
       <c r="F134" s="3">
-        <v>68.2</v>
+        <v>61.69</v>
       </c>
       <c r="L134" s="4"/>
       <c r="M134" s="4"/>
@@ -7038,7 +7039,8 @@
       <c r="X134" s="4"/>
       <c r="Y134" s="4"/>
       <c r="Z134" s="9">
-        <v>68.2</v>
+        <f>68.2-6.51</f>
+        <v>61.690000000000005</v>
       </c>
       <c r="AA134" s="4"/>
       <c r="AB134" s="4"/>
@@ -9012,7 +9014,7 @@
         <v>34</v>
       </c>
       <c r="F187" s="3">
-        <v>38.299999999999997</v>
+        <v>37.58</v>
       </c>
       <c r="L187" s="4"/>
       <c r="M187" s="4"/>
@@ -9029,7 +9031,7 @@
       <c r="X187" s="4"/>
       <c r="Y187" s="4"/>
       <c r="Z187" s="9">
-        <v>38.299999999999997</v>
+        <v>37.58</v>
       </c>
       <c r="AA187" s="4"/>
       <c r="AB187" s="4"/>

</xml_diff>